<commit_message>
Peak sponsorships: website pass on the top names (most public routes are charity budgets that exclude advertising: ask for marketing), two new ideas, Cheyenne Mountain Resort flagged as a possible competitor (Matthew 2026-10-21: 'go ahead and start the website pass')
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
+++ b/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
@@ -12,19 +12,21 @@
     <sheet name="Renewals (Peak sponsors)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Employers 400+" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="What others charge" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Ideas to borrow" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Wellhub" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Fact-check" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Pitch and tour invite" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Website pass" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Ideas to borrow" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Wellhub" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Fact-check" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Pitch and tour invite" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$Q$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Renewals (Peak sponsors)'!$A$1:$G$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Employers 400+'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'What others charge'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Ideas to borrow'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Wellhub'!$A$1:$C$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Fact-check'!$A$1:$D$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Website pass'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Ideas to borrow'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Wellhub'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Fact-check'!$A$1:$D$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -509,42 +511,173 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Ideas to borrow: what Springs Pickleball sells that Peak could. Wellhub: what Peak offers there, and ideas.</t>
+          <t>Website pass: what the free search found for the top names (most public routes are charity budgets: ask for marketing).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Route in: how to reach them. "To find" means the next step is finding the marketing or community contact (website, call the front desk, LinkedIn by hand).</t>
+          <t>Ideas to borrow: what Springs Pickleball sells that Peak could. Wellhub: what Peak offers there, and ideas.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Employers 400+: for group memberships and staff discounts. Counts with old years need confirming before you quote them.</t>
+          <t>Route in: how to reach them. "To find" means the next step is finding the marketing or community contact (website, call the front desk, LinkedIn by hand).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>What others charge: published prices from other venues, each checked at its source. Peak’s own prices are on top for comparison.</t>
+          <t>Employers 400+: for group memberships and staff discounts. Counts with old years need confirming before you quote them.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Fact-check: what was verified, corrected, and left out.</t>
+          <t>What others charge: published prices from other venues, each checked at its source. Peak’s own prices are on top for comparison.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Fact-check: what was verified, corrected, and left out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Nothing in this file has been sent to anyone.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Short pitch (for Brandon; check every fact with Peak before use)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Peak Pickleball has 24 indoor courts at Chapel Hills Mall. A court sponsorship puts your name on a court that players look at every time they play there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>We would like to show you the club. A 20-minute tour, any weekday, and you can see the courts, the crowd and where your name would go.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Tour invite (email draft; not sent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Subject: A 20-minute tour of Peak Pickleball</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Hi [first name],</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>I work with Peak Pickleball at Chapel Hills Mall: 24 indoor courts. We have a few court sponsorships open for [year] and I think [company] would be a good fit because [one line from the "Why they fit" column].</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Could I show you around for 20 minutes? Any weekday that suits you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>[Brandon’s name and number]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>- Tours sell: the price only comes up after they have seen the courts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>- Several companies set next year’s sponsorship budget in Q3 or Q4 (OCC closes on 30 Sep). Ask each one when its budget is set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>- Employers: lead with group memberships or a staff discount, not sponsorship. Peak is already on Wellhub: ask whether the company offers Wellhub before offering a second discount for the same thing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>- No member counts, visit numbers or follower counts in the pitch until Peak gives real ones.</t>
         </is>
       </c>
     </row>
@@ -886,12 +1019,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Cheyenne Mountain Resort</t>
+          <t>Molson Coors</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Resort</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -911,12 +1044,12 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -937,22 +1070,22 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Molson Coors</t>
+          <t>OrangeTheory</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Beverage</t>
+          <t>Fitness</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
         <v>6</v>
       </c>
       <c r="E7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>2</v>
@@ -962,17 +1095,17 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
+          <t>To find (franchise: the local owner decides)</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr"/>
@@ -988,22 +1121,22 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>OrangeTheory</t>
+          <t>Cheyenne Mountain Resort</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
+          <t>Resort</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>2</v>
@@ -1013,7 +1146,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1023,7 +1156,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>To find (franchise: the local owner decides)</t>
+          <t>To find</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr"/>
@@ -4342,7 +4475,310 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Public route found</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>What it means for Peak</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Kaiser Permanente</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Email communityco@kp.org (Colorado sponsorships; up to 6 weeks)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Its rules exclude "advertising activities" and team sponsorships: a court sign will not qualify. Only a community-health event (e.g. free beginner clinics) might.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://about.kaiserpermanente.org/community-health/communities-we-serve/colorado-community/sponsorships-conferences-and-community-service</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>UCHealth</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Community and government affairs, southern Colorado</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Its money goes out as grants to nonprofits. A sign at Peak is a marketing spend: ask for marketing, not community giving.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Ent Credit Union</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>CommunityAdvocacy@Ent.com is for nonprofit grants</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Ent says marketing sponsorships are handled separately, at the business level: ask for marketing. Ent is merging with Wings Credit Union.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ent.com/Community</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>BOK Financial</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Online charitable applications</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Its giving excludes "athletic programs". Bill Sullivan is listed as President &amp; CEO, Colorado Market: a marketing conversation, not a giving request.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://thestatement.bokf.com/Experts/Bill-Sullivan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Alpine Bank</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Event sponsorship form (2017, Denver office, written for nonprofits)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Stale and not for a for-profit venue. Ask a Colorado Springs branch who handles marketing.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.alpinebank.com/custom/fi/alpinebank/fb/disclosure/Sponsorship_Request_Form_Front-Range.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Cheyenne Mountain Resort</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Not looked for</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>A 2023 travel guide lists pickleball courts at the resort: possibly a competitor. Check before pitching.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>https://coloradoavidgolfer.com/colorado-getaways-2023-cheyenne-mountain-resort/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Molson Coors</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>No public route found</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Gives mostly in Golden and Denver and to disaster relief.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.molsoncoorsblog.com/node/11806</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Coca-Cola (Swire Coca-Cola, USA)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>No public route found</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Announced a $475M, 620,000 sq ft plant at Peak Innovation Park in Colorado Springs (Dec 2025), about 170 jobs: a local hook.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kktv.com/2025/12/11/swire-coca-cola-facility-coming-colorado-springs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Concept Restaurants</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>No marketing contact found</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>A Gazette Q&amp;A (undated) names co-owners Luke Travins and Dave Lux; ask at MacKenzie’s Chop House or Ritz Grill.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://gazette.com/?p=1156034</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>OrangeTheory</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Franchise: the studio owner decides</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Owner names found are from 2013 (Stetson Hills studio): ask the studio.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.franchising.com/amp/news/20131202_orangetheory_fitness_set_to_open_first_southern_co.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Media Group</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Not identified</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Nothing found under this name; ask the Sports Corp who it is.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Orthopedic Centers of Colorado (current Peak sponsor)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Outreach form; 1-866-506-7200; info@occ-ortho.com</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Open to "athletic partnerships"; proposals due 30 Sep, some exceptions. Already a Peak court sponsor: this is the renewal route.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://occ-ortho.com/community-outreach-and-sponsorship/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4364,82 +4800,106 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Bundle memberships into court sponsorships</t>
+          <t>Sell to marketing budgets, not charity</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Springs Pickleball’s $1,000/month Court Partner includes 4 memberships, paddles and gear. Peak’s $12,000 court could include staff memberships: it costs Peak little and the sponsor’s staff become players.</t>
+          <t>Most corporate "sponsorship request" pages are charity budgets for nonprofits, and several exclude advertising or athletics (Kaiser, BOK, Ent’s grants). A court sign at a for-profit club is advertising: Brandon needs the marketing or business-development person, and the pitch is reach and return, not giving.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Cheaper ways in</t>
+          <t>Look like Peak’s current sponsors</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Springs Pickleball starts at $250 (event tables) and $1,500 (a league season). Peak’s lowest published step is $12,000. A league, tournament or event-table tier lets small local businesses start, then move up.</t>
+          <t>Peak’s 28 sponsors are mostly local, owner-run businesses: car dealer, restaurants, home services, clinics, realtors, financial advisors. Owners decide fast. More of the same kind (other dealers, clinics, roofers, med spas near Chapel Hills) may close faster than big corporations.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Category exclusivity</t>
+          <t>Bundle memberships into court sponsorships</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Springs Pickleball sells it as an add-on: one bank, one hospital, one car dealer. Charge for it, or use it to close.</t>
+          <t>Springs Pickleball’s $1,000/month Court Partner includes 4 memberships, paddles and gear. Peak’s $12,000 court could include staff memberships: it costs Peak little and the sponsor’s staff become players.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Publish the audience</t>
+          <t>Cheaper ways in</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Springs Pickleball shows 20,000+ players, 4,000+ followers, 65+ at every Paddle Up night, 100–300 at events. Peak needs its own real numbers on its sponsor sheet (visits, members, event counts, followers).</t>
+          <t>Springs Pickleball starts at $250 (event tables) and $1,500 (a league season). Peak’s lowest published step is $12,000. A league, tournament or event-table tier lets small local businesses start, then move up.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Tournaments and livestream</t>
+          <t>Category exclusivity</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Springs Pickleball sells tournament tiers with livestream and social coverage. Peak’s national events are a bigger story: sell them as their own packages.</t>
+          <t>Springs Pickleball sells it as an add-on: one bank, one hospital, one car dealer. Charge for it, or use it to close.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>Publish the audience</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Springs Pickleball shows 20,000+ players, 4,000+ followers, 65+ at every Paddle Up night, 100–300 at events. Peak needs its own real numbers on its sponsor sheet (visits, members, event counts, followers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tournaments and livestream</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Springs Pickleball sells tournament tiers with livestream and social coverage. Peak’s national events are a bigger story: sell them as their own packages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>Socials as sponsor space</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Peak’s Instagram has 918 followers against Springs Pickleball’s 4,000+. Taking over and growing Peak’s socials is what makes posts, stories and video worth selling to sponsors.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4562,7 +5022,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5043,128 +5503,4 @@
   <autoFilter ref="A1:D21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Short pitch (for Brandon; check every fact with Peak before use)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Peak Pickleball has 24 indoor courts at Chapel Hills Mall. A court sponsorship puts your name on a court that players look at every time they play there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>We would like to show you the club. A 20-minute tour, any weekday, and you can see the courts, the crowd and where your name would go.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Tour invite (email draft; not sent)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Subject: A 20-minute tour of Peak Pickleball</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Hi [first name],</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>I work with Peak Pickleball at Chapel Hills Mall: 24 indoor courts. We have a few court sponsorships open for [year] and I think [company] would be a good fit because [one line from the "Why they fit" column].</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Could I show you around for 20 minutes? Any weekday that suits you.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>[Brandon’s name and number]</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>- Tours sell: the price only comes up after they have seen the courts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>- Several companies set next year’s sponsorship budget in Q3 or Q4 (OCC closes on 30 Sep). Ask each one when its budget is set.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>- Employers: lead with group memberships or a staff discount, not sponsorship. Peak is already on Wellhub: ask whether the company offers Wellhub before offering a second discount for the same thing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>- No member counts, visit numbers or follower counts in the pitch until Peak gives real ones.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Peak: Hunter's direct phone numbers carried into the desk and the Contacts tab (12 of the 39 have one); live seed updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
+++ b/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Renewals (Peak sponsors)'!$A$1:$G$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Employers 400+'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'What others charge'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Contacts (Hunter)'!$A$1:$I$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Contacts (Hunter)'!$A$1:$J$197</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Local lookalikes'!$A$1:$L$578</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Website pass'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Ideas to borrow'!$A$1:$B$9</definedName>
@@ -5099,7 +5099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I197"/>
+  <dimension ref="A1:J197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5111,6 +5111,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5159,6 +5160,11 @@
           <t>Pick</t>
         </is>
       </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -5198,6 +5204,11 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>+1 970 384 3216</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -5237,6 +5248,7 @@
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -5276,6 +5288,7 @@
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -5315,6 +5328,7 @@
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -5354,6 +5368,7 @@
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -5389,6 +5404,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -5428,6 +5444,7 @@
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -5467,6 +5484,7 @@
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -5506,6 +5524,7 @@
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -5545,6 +5564,7 @@
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -5588,6 +5608,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -5627,6 +5648,7 @@
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -5666,6 +5688,7 @@
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -5705,6 +5728,7 @@
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -5744,6 +5768,7 @@
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -5783,6 +5808,7 @@
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -5822,6 +5848,7 @@
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -5861,6 +5888,7 @@
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -5900,6 +5928,7 @@
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -5939,6 +5968,7 @@
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -5978,6 +6008,11 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>+1 719 584 4499</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -6017,6 +6052,11 @@
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>+1 720 848 7852</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -6056,6 +6096,11 @@
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>+1 303 956 0160</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -6091,6 +6136,11 @@
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>+1 720 316 7561</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -6130,6 +6180,11 @@
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>+1 307 421 9315</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -6169,6 +6224,7 @@
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -6204,6 +6260,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -6243,6 +6300,7 @@
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -6278,6 +6336,7 @@
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -6313,6 +6372,11 @@
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>+1 970 871 2522</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -6356,6 +6420,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -6395,6 +6460,7 @@
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -6434,6 +6500,7 @@
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -6473,6 +6540,7 @@
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -6512,6 +6580,11 @@
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>+1 801 816 5714</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -6551,6 +6624,7 @@
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -6590,6 +6664,7 @@
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -6629,6 +6704,7 @@
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -6668,6 +6744,7 @@
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -6707,6 +6784,7 @@
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -6750,6 +6828,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -6789,6 +6868,7 @@
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -6828,6 +6908,7 @@
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -6867,6 +6948,7 @@
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -6906,6 +6988,7 @@
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -6945,6 +7028,7 @@
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -6984,6 +7068,7 @@
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -7023,6 +7108,7 @@
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -7062,6 +7148,7 @@
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -7101,6 +7188,7 @@
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -7144,6 +7232,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -7179,6 +7268,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr"/>
       <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -7214,6 +7304,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr"/>
       <c r="I54" s="4" t="inlineStr"/>
+      <c r="J54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -7253,6 +7344,7 @@
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -7288,6 +7380,7 @@
       </c>
       <c r="H56" s="4" t="inlineStr"/>
       <c r="I56" s="4" t="inlineStr"/>
+      <c r="J56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -7327,6 +7420,7 @@
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -7366,6 +7460,7 @@
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr"/>
+      <c r="J58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -7405,6 +7500,7 @@
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -7444,6 +7540,11 @@
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr"/>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>+1 719 636 0142</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -7483,6 +7584,7 @@
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -7522,6 +7624,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -7557,6 +7660,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr"/>
       <c r="I63" s="4" t="inlineStr"/>
+      <c r="J63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -7592,6 +7696,11 @@
       </c>
       <c r="H64" s="4" t="inlineStr"/>
       <c r="I64" s="4" t="inlineStr"/>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>+1 918 594 7794</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -7627,6 +7736,7 @@
       </c>
       <c r="H65" s="4" t="inlineStr"/>
       <c r="I65" s="4" t="inlineStr"/>
+      <c r="J65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -7662,6 +7772,7 @@
       </c>
       <c r="H66" s="4" t="inlineStr"/>
       <c r="I66" s="4" t="inlineStr"/>
+      <c r="J66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -7697,6 +7808,11 @@
       </c>
       <c r="H67" s="4" t="inlineStr"/>
       <c r="I67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>+1 713 289 5876</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -7732,6 +7848,7 @@
       </c>
       <c r="H68" s="4" t="inlineStr"/>
       <c r="I68" s="4" t="inlineStr"/>
+      <c r="J68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -7767,6 +7884,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr"/>
       <c r="I69" s="4" t="inlineStr"/>
+      <c r="J69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -7802,6 +7920,7 @@
       </c>
       <c r="H70" s="4" t="inlineStr"/>
       <c r="I70" s="4" t="inlineStr"/>
+      <c r="J70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -7837,6 +7956,11 @@
       </c>
       <c r="H71" s="4" t="inlineStr"/>
       <c r="I71" s="4" t="inlineStr"/>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>+1 214 576 0878</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -7880,6 +8004,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -7919,6 +8044,7 @@
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr"/>
+      <c r="J73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -7954,6 +8080,7 @@
       </c>
       <c r="H74" s="4" t="inlineStr"/>
       <c r="I74" s="4" t="inlineStr"/>
+      <c r="J74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -7997,6 +8124,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -8036,6 +8164,7 @@
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr"/>
+      <c r="J76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -8075,6 +8204,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -8110,6 +8240,7 @@
       </c>
       <c r="H78" s="4" t="inlineStr"/>
       <c r="I78" s="4" t="inlineStr"/>
+      <c r="J78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -8145,6 +8276,7 @@
       </c>
       <c r="H79" s="4" t="inlineStr"/>
       <c r="I79" s="4" t="inlineStr"/>
+      <c r="J79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -8188,6 +8320,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -8227,6 +8360,7 @@
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr"/>
+      <c r="J81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -8266,6 +8400,7 @@
         </is>
       </c>
       <c r="I82" s="4" t="inlineStr"/>
+      <c r="J82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -8305,6 +8440,7 @@
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr"/>
+      <c r="J83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -8344,6 +8480,7 @@
         </is>
       </c>
       <c r="I84" s="4" t="inlineStr"/>
+      <c r="J84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -8383,6 +8520,7 @@
         </is>
       </c>
       <c r="I85" s="4" t="inlineStr"/>
+      <c r="J85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -8422,6 +8560,7 @@
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr"/>
+      <c r="J86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -8457,6 +8596,7 @@
       </c>
       <c r="H87" s="4" t="inlineStr"/>
       <c r="I87" s="4" t="inlineStr"/>
+      <c r="J87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -8496,6 +8636,7 @@
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr"/>
+      <c r="J88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -8535,6 +8676,7 @@
         </is>
       </c>
       <c r="I89" s="4" t="inlineStr"/>
+      <c r="J89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -8574,6 +8716,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -8617,6 +8760,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -8656,6 +8800,7 @@
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr"/>
+      <c r="J92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -8695,6 +8840,7 @@
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr"/>
+      <c r="J93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -8734,6 +8880,7 @@
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr"/>
+      <c r="J94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -8773,6 +8920,7 @@
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr"/>
+      <c r="J95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -8812,6 +8960,7 @@
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr"/>
+      <c r="J96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -8851,6 +9000,7 @@
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr"/>
+      <c r="J97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -8890,6 +9040,11 @@
         </is>
       </c>
       <c r="I98" s="4" t="inlineStr"/>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>+1 214 523 2780</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -8929,6 +9084,7 @@
         </is>
       </c>
       <c r="I99" s="4" t="inlineStr"/>
+      <c r="J99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -8968,6 +9124,7 @@
         </is>
       </c>
       <c r="I100" s="4" t="inlineStr"/>
+      <c r="J100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -9007,6 +9164,11 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>+1 254 742 3637</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -9046,6 +9208,7 @@
         </is>
       </c>
       <c r="I102" s="4" t="inlineStr"/>
+      <c r="J102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -9085,6 +9248,7 @@
         </is>
       </c>
       <c r="I103" s="4" t="inlineStr"/>
+      <c r="J103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -9124,6 +9288,7 @@
         </is>
       </c>
       <c r="I104" s="4" t="inlineStr"/>
+      <c r="J104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -9163,6 +9328,7 @@
         </is>
       </c>
       <c r="I105" s="4" t="inlineStr"/>
+      <c r="J105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -9198,6 +9364,7 @@
       </c>
       <c r="H106" s="4" t="inlineStr"/>
       <c r="I106" s="4" t="inlineStr"/>
+      <c r="J106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -9237,6 +9404,7 @@
         </is>
       </c>
       <c r="I107" s="4" t="inlineStr"/>
+      <c r="J107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -9276,6 +9444,7 @@
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr"/>
+      <c r="J108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -9315,6 +9484,7 @@
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr"/>
+      <c r="J109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -9354,6 +9524,7 @@
         </is>
       </c>
       <c r="I110" s="4" t="inlineStr"/>
+      <c r="J110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -9397,6 +9568,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -9436,6 +9608,7 @@
         </is>
       </c>
       <c r="I112" s="4" t="inlineStr"/>
+      <c r="J112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -9475,6 +9648,7 @@
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr"/>
+      <c r="J113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -9514,6 +9688,7 @@
         </is>
       </c>
       <c r="I114" s="4" t="inlineStr"/>
+      <c r="J114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -9553,6 +9728,7 @@
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr"/>
+      <c r="J115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -9592,6 +9768,7 @@
         </is>
       </c>
       <c r="I116" s="4" t="inlineStr"/>
+      <c r="J116" s="4" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -9631,6 +9808,7 @@
         </is>
       </c>
       <c r="I117" s="4" t="inlineStr"/>
+      <c r="J117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -9670,6 +9848,7 @@
         </is>
       </c>
       <c r="I118" s="4" t="inlineStr"/>
+      <c r="J118" s="4" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -9709,6 +9888,7 @@
         </is>
       </c>
       <c r="I119" s="4" t="inlineStr"/>
+      <c r="J119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -9748,6 +9928,11 @@
         </is>
       </c>
       <c r="I120" s="4" t="inlineStr"/>
+      <c r="J120" s="4" t="inlineStr">
+        <is>
+          <t>+1 416 201 9995</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -9787,6 +9972,11 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J121" s="4" t="inlineStr">
+        <is>
+          <t>+1 480 718 0119</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -9826,6 +10016,7 @@
         </is>
       </c>
       <c r="I122" s="4" t="inlineStr"/>
+      <c r="J122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -9865,6 +10056,7 @@
         </is>
       </c>
       <c r="I123" s="4" t="inlineStr"/>
+      <c r="J123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -9904,6 +10096,7 @@
         </is>
       </c>
       <c r="I124" s="4" t="inlineStr"/>
+      <c r="J124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -9943,6 +10136,7 @@
         </is>
       </c>
       <c r="I125" s="4" t="inlineStr"/>
+      <c r="J125" s="4" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -9978,6 +10172,7 @@
       </c>
       <c r="H126" s="4" t="inlineStr"/>
       <c r="I126" s="4" t="inlineStr"/>
+      <c r="J126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -10013,6 +10208,7 @@
       </c>
       <c r="H127" s="4" t="inlineStr"/>
       <c r="I127" s="4" t="inlineStr"/>
+      <c r="J127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -10048,6 +10244,7 @@
       </c>
       <c r="H128" s="4" t="inlineStr"/>
       <c r="I128" s="4" t="inlineStr"/>
+      <c r="J128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -10083,6 +10280,7 @@
       </c>
       <c r="H129" s="4" t="inlineStr"/>
       <c r="I129" s="4" t="inlineStr"/>
+      <c r="J129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -10118,6 +10316,7 @@
       </c>
       <c r="H130" s="4" t="inlineStr"/>
       <c r="I130" s="4" t="inlineStr"/>
+      <c r="J130" s="4" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -10161,6 +10360,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -10200,6 +10400,7 @@
         </is>
       </c>
       <c r="I132" s="4" t="inlineStr"/>
+      <c r="J132" s="4" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -10239,6 +10440,7 @@
         </is>
       </c>
       <c r="I133" s="4" t="inlineStr"/>
+      <c r="J133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -10278,6 +10480,7 @@
         </is>
       </c>
       <c r="I134" s="4" t="inlineStr"/>
+      <c r="J134" s="4" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -10317,6 +10520,7 @@
         </is>
       </c>
       <c r="I135" s="4" t="inlineStr"/>
+      <c r="J135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -10356,6 +10560,7 @@
         </is>
       </c>
       <c r="I136" s="4" t="inlineStr"/>
+      <c r="J136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -10391,6 +10596,7 @@
       </c>
       <c r="H137" s="4" t="inlineStr"/>
       <c r="I137" s="4" t="inlineStr"/>
+      <c r="J137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -10426,6 +10632,11 @@
       </c>
       <c r="H138" s="4" t="inlineStr"/>
       <c r="I138" s="4" t="inlineStr"/>
+      <c r="J138" s="4" t="inlineStr">
+        <is>
+          <t>+1 719 756 2288</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -10461,6 +10672,7 @@
       </c>
       <c r="H139" s="4" t="inlineStr"/>
       <c r="I139" s="4" t="inlineStr"/>
+      <c r="J139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -10500,6 +10712,7 @@
         </is>
       </c>
       <c r="I140" s="4" t="inlineStr"/>
+      <c r="J140" s="4" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -10543,6 +10756,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -10578,6 +10792,7 @@
       </c>
       <c r="H142" s="4" t="inlineStr"/>
       <c r="I142" s="4" t="inlineStr"/>
+      <c r="J142" s="4" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -10617,6 +10832,7 @@
         </is>
       </c>
       <c r="I143" s="4" t="inlineStr"/>
+      <c r="J143" s="4" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -10656,6 +10872,7 @@
         </is>
       </c>
       <c r="I144" s="4" t="inlineStr"/>
+      <c r="J144" s="4" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -10695,6 +10912,7 @@
         </is>
       </c>
       <c r="I145" s="4" t="inlineStr"/>
+      <c r="J145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -10734,6 +10952,7 @@
         </is>
       </c>
       <c r="I146" s="4" t="inlineStr"/>
+      <c r="J146" s="4" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -10773,6 +10992,7 @@
         </is>
       </c>
       <c r="I147" s="4" t="inlineStr"/>
+      <c r="J147" s="4" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -10812,6 +11032,7 @@
         </is>
       </c>
       <c r="I148" s="4" t="inlineStr"/>
+      <c r="J148" s="4" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -10851,6 +11072,7 @@
         </is>
       </c>
       <c r="I149" s="4" t="inlineStr"/>
+      <c r="J149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -10886,6 +11108,7 @@
       </c>
       <c r="H150" s="4" t="inlineStr"/>
       <c r="I150" s="4" t="inlineStr"/>
+      <c r="J150" s="4" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -10925,6 +11148,11 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J151" s="4" t="inlineStr">
+        <is>
+          <t>+1 440 395 2222</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -10960,6 +11188,11 @@
       </c>
       <c r="H152" s="4" t="inlineStr"/>
       <c r="I152" s="4" t="inlineStr"/>
+      <c r="J152" s="4" t="inlineStr">
+        <is>
+          <t>+1 440 603 2100</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -10999,6 +11232,7 @@
         </is>
       </c>
       <c r="I153" s="4" t="inlineStr"/>
+      <c r="J153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -11034,6 +11268,7 @@
       </c>
       <c r="H154" s="4" t="inlineStr"/>
       <c r="I154" s="4" t="inlineStr"/>
+      <c r="J154" s="4" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -11073,6 +11308,7 @@
         </is>
       </c>
       <c r="I155" s="4" t="inlineStr"/>
+      <c r="J155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -11108,6 +11344,7 @@
       </c>
       <c r="H156" s="4" t="inlineStr"/>
       <c r="I156" s="4" t="inlineStr"/>
+      <c r="J156" s="4" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -11143,6 +11380,11 @@
       </c>
       <c r="H157" s="4" t="inlineStr"/>
       <c r="I157" s="4" t="inlineStr"/>
+      <c r="J157" s="4" t="inlineStr">
+        <is>
+          <t>+1 800 274 4055</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -11178,6 +11420,11 @@
       </c>
       <c r="H158" s="4" t="inlineStr"/>
       <c r="I158" s="4" t="inlineStr"/>
+      <c r="J158" s="4" t="inlineStr">
+        <is>
+          <t>+1 800 274 4055</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -11213,6 +11460,7 @@
       </c>
       <c r="H159" s="4" t="inlineStr"/>
       <c r="I159" s="4" t="inlineStr"/>
+      <c r="J159" s="4" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -11248,6 +11496,11 @@
       </c>
       <c r="H160" s="4" t="inlineStr"/>
       <c r="I160" s="4" t="inlineStr"/>
+      <c r="J160" s="4" t="inlineStr">
+        <is>
+          <t>+1 419 722 9316</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -11291,6 +11544,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J161" s="4" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -11330,6 +11584,11 @@
         </is>
       </c>
       <c r="I162" s="4" t="inlineStr"/>
+      <c r="J162" s="4" t="inlineStr">
+        <is>
+          <t>+1 916 717 1072</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -11369,6 +11628,11 @@
         </is>
       </c>
       <c r="I163" s="4" t="inlineStr"/>
+      <c r="J163" s="4" t="inlineStr">
+        <is>
+          <t>+1 210 290 1748</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -11408,6 +11672,7 @@
         </is>
       </c>
       <c r="I164" s="4" t="inlineStr"/>
+      <c r="J164" s="4" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -11443,6 +11708,11 @@
       </c>
       <c r="H165" s="4" t="inlineStr"/>
       <c r="I165" s="4" t="inlineStr"/>
+      <c r="J165" s="4" t="inlineStr">
+        <is>
+          <t>+1 210 498 7578</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -11478,6 +11748,11 @@
       </c>
       <c r="H166" s="4" t="inlineStr"/>
       <c r="I166" s="4" t="inlineStr"/>
+      <c r="J166" s="4" t="inlineStr">
+        <is>
+          <t>+1 210 531 8722</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -11513,6 +11788,7 @@
       </c>
       <c r="H167" s="4" t="inlineStr"/>
       <c r="I167" s="4" t="inlineStr"/>
+      <c r="J167" s="4" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -11552,6 +11828,11 @@
         </is>
       </c>
       <c r="I168" s="4" t="inlineStr"/>
+      <c r="J168" s="4" t="inlineStr">
+        <is>
+          <t>+1 210 498 1479</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -11587,6 +11868,7 @@
       </c>
       <c r="H169" s="4" t="inlineStr"/>
       <c r="I169" s="4" t="inlineStr"/>
+      <c r="J169" s="4" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -11622,6 +11904,7 @@
       </c>
       <c r="H170" s="4" t="inlineStr"/>
       <c r="I170" s="4" t="inlineStr"/>
+      <c r="J170" s="4" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -11665,6 +11948,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J171" s="4" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -11700,6 +11984,7 @@
       </c>
       <c r="H172" s="4" t="inlineStr"/>
       <c r="I172" s="4" t="inlineStr"/>
+      <c r="J172" s="4" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -11743,6 +12028,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -11786,6 +12072,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J174" s="4" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -11821,6 +12108,7 @@
       </c>
       <c r="H175" s="4" t="inlineStr"/>
       <c r="I175" s="4" t="inlineStr"/>
+      <c r="J175" s="4" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -11860,6 +12148,7 @@
         </is>
       </c>
       <c r="I176" s="4" t="inlineStr"/>
+      <c r="J176" s="4" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -11895,6 +12184,7 @@
       </c>
       <c r="H177" s="4" t="inlineStr"/>
       <c r="I177" s="4" t="inlineStr"/>
+      <c r="J177" s="4" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -11930,6 +12220,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J178" s="4" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -11965,6 +12256,7 @@
       </c>
       <c r="H179" s="4" t="inlineStr"/>
       <c r="I179" s="4" t="inlineStr"/>
+      <c r="J179" s="4" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -12004,6 +12296,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J180" s="4" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -12043,6 +12336,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J181" s="4" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -12074,6 +12368,7 @@
       </c>
       <c r="H182" s="4" t="inlineStr"/>
       <c r="I182" s="4" t="inlineStr"/>
+      <c r="J182" s="4" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -12109,6 +12404,7 @@
       </c>
       <c r="H183" s="4" t="inlineStr"/>
       <c r="I183" s="4" t="inlineStr"/>
+      <c r="J183" s="4" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -12144,6 +12440,7 @@
       </c>
       <c r="H184" s="4" t="inlineStr"/>
       <c r="I184" s="4" t="inlineStr"/>
+      <c r="J184" s="4" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -12183,6 +12480,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J185" s="4" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -12222,6 +12520,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J186" s="4" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -12261,6 +12560,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J187" s="4" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -12296,6 +12596,7 @@
       </c>
       <c r="H188" s="4" t="inlineStr"/>
       <c r="I188" s="4" t="inlineStr"/>
+      <c r="J188" s="4" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -12335,6 +12636,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J189" s="4" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -12370,6 +12672,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J190" s="4" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -12409,6 +12712,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J191" s="4" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -12448,6 +12752,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J192" s="4" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
@@ -12487,6 +12792,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J193" s="4" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -12526,6 +12832,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J194" s="4" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
@@ -12565,6 +12872,7 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J195" s="4" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -12600,6 +12908,7 @@
       </c>
       <c r="H196" s="4" t="inlineStr"/>
       <c r="I196" s="4" t="inlineStr"/>
+      <c r="J196" s="4" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -12639,9 +12948,10 @@
           <t>Ask for first</t>
         </is>
       </c>
+      <c r="J197" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I197"/>
+  <autoFilter ref="A1:J197"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Peak: main and local phone lines for 16 of the 39 (own sites, an SEC filing or consistent listings; conflicts left out), each with where it came from; in the desk (live) and the Sponsor leads tab (Matthew 2026-10-21)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
+++ b/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
@@ -21,7 +21,7 @@
     <sheet name="Pitch and tour invite" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$Q$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$S$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Renewals (Peak sponsors)'!$A$1:$G$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Employers 400+'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'What others charge'!$A$1:$H$13</definedName>
@@ -1316,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1424,6 +1424,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Main / local phone</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Phone source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
@@ -1475,6 +1485,8 @@
       <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="4" t="inlineStr"/>
+      <c r="S2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1530,6 +1542,8 @@
       <c r="O3" s="5" t="inlineStr"/>
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="4" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -1585,6 +1599,16 @@
       <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>719-421-7600</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs branch, 90 S Cascade Ave, Ste 100 · https://www.alpinebank.com/locations/colorado-springs.html</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -1636,6 +1660,16 @@
       <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>303-863-4270</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>Colorado commercial banking (no Colorado Springs office listed) · https://bokfinancial.com/location-and-contact-us/additional-contact-information/CO</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -1687,6 +1721,16 @@
       <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr"/>
       <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>303-279-6565</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>head office, Golden · SEC EDGAR filing, business phone</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -1738,6 +1782,8 @@
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -1789,6 +1835,16 @@
       <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>719-583-4000</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -1840,6 +1896,8 @@
       <c r="O9" s="5" t="inlineStr"/>
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -1891,6 +1949,8 @@
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1942,6 +2002,16 @@
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>719-257-5745</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -1993,6 +2063,16 @@
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>719-330-7448</t>
+        </is>
+      </c>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs) · https://www.visitcos.com/directory/colorado-media-group-real-estate/</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2044,6 +2124,16 @@
       <c r="O13" s="5" t="inlineStr"/>
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>719-471-8183</t>
+        </is>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>main line; email info@cscedc.com · https://coloradospringschamberedc.com/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -2095,6 +2185,16 @@
       <c r="O14" s="5" t="inlineStr"/>
       <c r="P14" s="5" t="inlineStr"/>
       <c r="Q14" s="5" t="inlineStr"/>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>719-635-3536</t>
+        </is>
+      </c>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -2146,6 +2246,16 @@
       <c r="O15" s="5" t="inlineStr"/>
       <c r="P15" s="5" t="inlineStr"/>
       <c r="Q15" s="5" t="inlineStr"/>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>719-593-2700</t>
+        </is>
+      </c>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -2197,6 +2307,16 @@
       <c r="O16" s="5" t="inlineStr"/>
       <c r="P16" s="5" t="inlineStr"/>
       <c r="Q16" s="5" t="inlineStr"/>
+      <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>800-525-9623</t>
+        </is>
+      </c>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -2248,6 +2368,8 @@
       <c r="O17" s="5" t="inlineStr"/>
       <c r="P17" s="5" t="inlineStr"/>
       <c r="Q17" s="5" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -2299,6 +2421,8 @@
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
       <c r="Q18" s="5" t="inlineStr"/>
+      <c r="R18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -2350,6 +2474,8 @@
       <c r="O19" s="5" t="inlineStr"/>
       <c r="P19" s="5" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr"/>
+      <c r="R19" s="4" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -2401,6 +2527,16 @@
       <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
+      <c r="R20" s="4" t="inlineStr">
+        <is>
+          <t>719-278-5600</t>
+        </is>
+      </c>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -2452,6 +2588,16 @@
       <c r="O21" s="5" t="inlineStr"/>
       <c r="P21" s="5" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="4" t="inlineStr">
+        <is>
+          <t>719-476-1645</t>
+        </is>
+      </c>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -2503,6 +2649,16 @@
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>844-844-4432</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -2554,6 +2710,16 @@
       <c r="O23" s="5" t="inlineStr"/>
       <c r="P23" s="5" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>719-964-1798</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -2605,6 +2771,8 @@
       <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr"/>
       <c r="Q24" s="5" t="inlineStr"/>
+      <c r="R24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2656,6 +2824,8 @@
       <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
       <c r="Q25" s="5" t="inlineStr"/>
+      <c r="R25" s="4" t="inlineStr"/>
+      <c r="S25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -2707,6 +2877,8 @@
       <c r="O26" s="5" t="inlineStr"/>
       <c r="P26" s="5" t="inlineStr"/>
       <c r="Q26" s="5" t="inlineStr"/>
+      <c r="R26" s="4" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -2758,6 +2930,8 @@
       <c r="O27" s="5" t="inlineStr"/>
       <c r="P27" s="5" t="inlineStr"/>
       <c r="Q27" s="5" t="inlineStr"/>
+      <c r="R27" s="4" t="inlineStr"/>
+      <c r="S27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -2809,6 +2983,8 @@
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="4" t="inlineStr"/>
+      <c r="S28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -2860,6 +3036,8 @@
       <c r="O29" s="5" t="inlineStr"/>
       <c r="P29" s="5" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr"/>
+      <c r="R29" s="4" t="inlineStr"/>
+      <c r="S29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -2911,6 +3089,8 @@
       <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="inlineStr"/>
       <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="4" t="inlineStr"/>
+      <c r="S30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -2962,6 +3142,16 @@
       <c r="O31" s="5" t="inlineStr"/>
       <c r="P31" s="5" t="inlineStr"/>
       <c r="Q31" s="5" t="inlineStr"/>
+      <c r="R31" s="4" t="inlineStr">
+        <is>
+          <t>970-690-7709</t>
+        </is>
+      </c>
+      <c r="S31" s="4" t="inlineStr">
+        <is>
+          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -3013,6 +3203,8 @@
       <c r="O32" s="5" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr"/>
       <c r="Q32" s="5" t="inlineStr"/>
+      <c r="R32" s="4" t="inlineStr"/>
+      <c r="S32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -3064,6 +3256,8 @@
       <c r="O33" s="5" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
       <c r="Q33" s="5" t="inlineStr"/>
+      <c r="R33" s="4" t="inlineStr"/>
+      <c r="S33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3115,6 +3309,8 @@
       <c r="O34" s="5" t="inlineStr"/>
       <c r="P34" s="5" t="inlineStr"/>
       <c r="Q34" s="5" t="inlineStr"/>
+      <c r="R34" s="4" t="inlineStr"/>
+      <c r="S34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -3166,6 +3362,8 @@
       <c r="O35" s="5" t="inlineStr"/>
       <c r="P35" s="5" t="inlineStr"/>
       <c r="Q35" s="5" t="inlineStr"/>
+      <c r="R35" s="4" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3217,6 +3415,8 @@
       <c r="O36" s="5" t="inlineStr"/>
       <c r="P36" s="5" t="inlineStr"/>
       <c r="Q36" s="5" t="inlineStr"/>
+      <c r="R36" s="4" t="inlineStr"/>
+      <c r="S36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3268,6 +3468,16 @@
       <c r="O37" s="5" t="inlineStr"/>
       <c r="P37" s="5" t="inlineStr"/>
       <c r="Q37" s="5" t="inlineStr"/>
+      <c r="R37" s="4" t="inlineStr">
+        <is>
+          <t>719-231-5353</t>
+        </is>
+      </c>
+      <c r="S37" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -3319,6 +3529,8 @@
       <c r="O38" s="5" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr"/>
       <c r="Q38" s="5" t="inlineStr"/>
+      <c r="R38" s="4" t="inlineStr"/>
+      <c r="S38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -3370,6 +3582,8 @@
       <c r="O39" s="5" t="inlineStr"/>
       <c r="P39" s="5" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr"/>
+      <c r="R39" s="4" t="inlineStr"/>
+      <c r="S39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -3421,9 +3635,11 @@
       <c r="O40" s="5" t="inlineStr"/>
       <c r="P40" s="5" t="inlineStr"/>
       <c r="Q40" s="5" t="inlineStr"/>
+      <c r="R40" s="4" t="inlineStr"/>
+      <c r="S40" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q40"/>
+  <autoFilter ref="A1:S40"/>
   <dataValidations count="1">
     <dataValidation sqref="M2:M40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,Emailed,Called,Tour booked,Toured,Proposal sent,Signed,Not now,No"</formula1>

</xml_diff>

<commit_message>
Peak leads ordered by score plus a point each for an email and a phone (Matthew 2026-10-21); best email and best phone shown on the Sponsor leads tab; Kaiser's and the Chamber's inboxes on the Contacts tab; the desk gets the same order, email/phone marks and a Score-only switch (live)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
+++ b/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
@@ -21,11 +21,11 @@
     <sheet name="Pitch and tour invite" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$S$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$V$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Renewals (Peak sponsors)'!$A$1:$G$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Employers 400+'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'What others charge'!$A$1:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Contacts (Hunter)'!$A$1:$J$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Contacts (Hunter)'!$A$1:$J$199</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Local lookalikes'!$A$1:$L$578</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Website pass'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Ideas to borrow'!$A$1:$B$9</definedName>
@@ -1316,32 +1316,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:V40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="58" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="44" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="58" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
     <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>Order</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -1356,80 +1361,95 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
+          <t>Best email</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Best phone</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Order points (score + email + phone)</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
           <t>Score /9</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Fit /3</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Money /3</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Sponsors sport /2</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Near Peak /1</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Why they fit</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Route in</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Route link</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Contact (name, role)</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Email / phone</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Next step / date</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Main / local phone</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Phone source</t>
         </is>
@@ -1449,44 +1469,53 @@
           <t>Health insurer / care</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>communityco@kp.org (Colorado community sponsorships, Sponsorship inbox (rules exclude advertising))</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Paid sponsor of the Colorado Chamber’s 2024 pickleball tournament (Pickle Hour and awards) at the Broadmoor.</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>To find (statewide marketing; check for a Colorado Springs community contact)</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr"/>
       <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="4" t="inlineStr"/>
-      <c r="S2" s="4" t="inlineStr"/>
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr"/>
+      <c r="T2" s="5" t="inlineStr"/>
+      <c r="U2" s="4" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1502,48 +1531,61 @@
           <t>Hospital system</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>todd.seip@uchealth.org (Todd Seip, Director Of Public Relations)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>+1 719 584 4499 (Todd Seip)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>No. 4 employer in El Paso County (7,050 staff, 2024). Gives through community grants (southern Colorado grants announced in UCHealth news).</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>https://epc-assets.elpasoco.com/wp-content/uploads/sites/2/2024-ACFR-FINAL-reduced-size.pdf ; https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Community and government affairs, southern Colorado (the senior director is named in UCHealth news releases). Also an employee-membership target (see Employers).</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr"/>
-      <c r="N3" s="5" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr"/>
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="4" t="inlineStr"/>
-      <c r="S3" s="4" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="4" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -1559,52 +1601,65 @@
           <t>Bank</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>alansandberg@alpinebank.com (Alan Sandberg, Director Of Marketing)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>719-421-7600 (Colorado Springs branch, 90 S Cascade Ave, Ste 100)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Front Range sponsorship request form (to its Denver office; asks 60 days ahead). The form may be dated: confirm the current contact first.</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>https://www.alpinebank.com/custom/fi/alpinebank/fb/disclosure/Sponsorship_Request_Form_Front-Range.pdf</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr"/>
+      <c r="T4" s="5" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>719-421-7600</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs branch, 90 S Cascade Ave, Ste 100 · https://www.alpinebank.com/locations/colorado-springs.html</t>
         </is>
@@ -1624,48 +1679,61 @@
           <t>Bank</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ggerst@bokf.com (Gilbert Gerst, Senior Vice President Community Development)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>303-863-4270 (Colorado commercial banking (no Colorado Springs office listed))</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr"/>
-      <c r="N5" s="5" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="4" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="5" t="inlineStr"/>
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>303-863-4270</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="V5" s="4" t="inlineStr">
         <is>
           <t>Colorado commercial banking (no Colorado Springs office listed) · https://bokfinancial.com/location-and-contact-us/additional-contact-information/CO</t>
         </is>
@@ -1685,48 +1753,61 @@
           <t>Beverage</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>meghan.means@molsoncoors.com (Meghan Means, Marketing Director)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>303-279-6565 (head office, Golden)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr"/>
       <c r="Q6" s="5" t="inlineStr"/>
-      <c r="R6" s="4" t="inlineStr">
+      <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr"/>
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>303-279-6565</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>head office, Golden · SEC EDGAR filing, business phone</t>
         </is>
@@ -1746,44 +1827,53 @@
           <t>Fitness</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>memberservices@orangetheory.com (General inbox)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>To find (franchise: the local owner decides)</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr"/>
-      <c r="O7" s="5" t="inlineStr"/>
+      <c r="O7" s="4" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
-      <c r="R7" s="4" t="inlineStr"/>
-      <c r="S7" s="4" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="inlineStr"/>
+      <c r="U7" s="4" t="inlineStr"/>
+      <c r="V7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -1791,58 +1881,71 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Cheyenne Mountain Resort</t>
+          <t>Coca-Cola</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Resort</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
+          <t>Beverage</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>apopescu@swirecc.com (Andrei Popescu, Marketing Director)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>719-257-5745 (Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="H8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Also a pouring-rights deal for Peak’s snack bar, if Peak has one.</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
-      <c r="O8" s="5" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>719-583-4000</t>
-        </is>
-      </c>
-      <c r="S8" s="4" t="inlineStr">
-        <is>
-          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
+      <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" s="5" t="inlineStr"/>
+      <c r="T8" s="5" t="inlineStr"/>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>719-257-5745</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
         </is>
       </c>
     </row>
@@ -1852,52 +1955,73 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Chord Energy</t>
+          <t>Colorado Media Group</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>dhobbs@coloradomediagroup.com (Dirk Hobbs, Division Manager)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>719-330-7448 (publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs))</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="H9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner, as above.</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr"/>
-      <c r="O9" s="5" t="inlineStr"/>
+      <c r="O9" s="4" t="inlineStr"/>
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
-      <c r="R9" s="4" t="inlineStr"/>
-      <c r="S9" s="4" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" s="5" t="inlineStr"/>
+      <c r="T9" s="5" t="inlineStr"/>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>719-330-7448</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs) · https://www.visitcos.com/directory/colorado-media-group-real-estate/</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -1905,52 +2029,73 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Climax Molybdenum</t>
+          <t>Colorado Springs Chamber &amp; EDC</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Mining</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
+          <t>Business network</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>info@cscedc.com (General inbox)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>719-471-8183 (main line)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="H10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Introductions to members and a venue for a member event at Peak.</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr"/>
-      <c r="O10" s="5" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
-      <c r="R10" s="4" t="inlineStr"/>
-      <c r="S10" s="4" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="5" t="inlineStr"/>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>719-471-8183</t>
+        </is>
+      </c>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>main line; email info@cscedc.com · https://coloradospringschamberedc.com/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1958,58 +2103,71 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Coca-Cola</t>
+          <t>Concept Restaurants</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Beverage</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="n">
+          <t>Restaurant group</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>erin@conceptrestaurants.com (Erin Copeland, Vice President of Marketing)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>719-635-3536 (MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A))</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Also a pouring-rights deal for Peak’s snack bar, if Peak has one.</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr"/>
-      <c r="N11" s="5" t="inlineStr"/>
-      <c r="O11" s="5" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
-      <c r="R11" s="4" t="inlineStr">
-        <is>
-          <t>719-257-5745</t>
-        </is>
-      </c>
-      <c r="S11" s="4" t="inlineStr">
-        <is>
-          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
+      <c r="R11" s="5" t="inlineStr"/>
+      <c r="S11" s="5" t="inlineStr"/>
+      <c r="T11" s="5" t="inlineStr"/>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>719-635-3536</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
         </is>
       </c>
     </row>
@@ -2019,58 +2177,71 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Colorado Media Group</t>
+          <t>Cumulus Media</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
+          <t>Radio</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>james.robinson@cumulus.com (James Robinson, Vice President, Marketing)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>719-593-2700 (Colorado Springs stations, 6805 Corporate Dr #130)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner, as above.</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="inlineStr"/>
-      <c r="O12" s="5" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
-      <c r="R12" s="4" t="inlineStr">
-        <is>
-          <t>719-330-7448</t>
-        </is>
-      </c>
-      <c r="S12" s="4" t="inlineStr">
-        <is>
-          <t>publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs) · https://www.visitcos.com/directory/colorado-media-group-real-estate/</t>
+      <c r="R12" s="5" t="inlineStr"/>
+      <c r="S12" s="5" t="inlineStr"/>
+      <c r="T12" s="5" t="inlineStr"/>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>719-593-2700</t>
+        </is>
+      </c>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
         </is>
       </c>
     </row>
@@ -2080,58 +2251,71 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Chamber &amp; EDC</t>
+          <t>Ent Credit Union</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
+          <t>Credit union</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>kutermoehlen@ent.com (Kelly Utermoehlen, Director of Internal Communications)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>800-525-9623 (main line)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Introductions to members and a venue for a member event at Peak.</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Headquartered in Colorado Springs; about 1,300 staff (Gazette, 2021). Big local sponsor profile.</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Gazette 2021 (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="5" t="inlineStr"/>
-      <c r="N13" s="5" t="inlineStr"/>
-      <c r="O13" s="5" t="inlineStr"/>
+      <c r="O13" s="4" t="inlineStr"/>
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
-      <c r="R13" s="4" t="inlineStr">
-        <is>
-          <t>719-471-8183</t>
-        </is>
-      </c>
-      <c r="S13" s="4" t="inlineStr">
-        <is>
-          <t>main line; email info@cscedc.com · https://coloradospringschamberedc.com/contact/</t>
+      <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" s="5" t="inlineStr"/>
+      <c r="T13" s="5" t="inlineStr"/>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>800-525-9623</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
         </is>
       </c>
     </row>
@@ -2141,60 +2325,65 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Concept Restaurants</t>
+          <t>McLane Company</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Restaurant group</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
+          <t>Distribution</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>tom.sicola@mclaneco.com (Tom Sicola, Vp Of Marketing)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>+1 254 742 3637 (Tom Sicola)</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr"/>
-      <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr"/>
-      <c r="O14" s="5" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
       <c r="P14" s="5" t="inlineStr"/>
       <c r="Q14" s="5" t="inlineStr"/>
-      <c r="R14" s="4" t="inlineStr">
-        <is>
-          <t>719-635-3536</t>
-        </is>
-      </c>
-      <c r="S14" s="4" t="inlineStr">
-        <is>
-          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
-        </is>
-      </c>
+      <c r="R14" s="5" t="inlineStr"/>
+      <c r="S14" s="5" t="inlineStr"/>
+      <c r="T14" s="5" t="inlineStr"/>
+      <c r="U14" s="4" t="inlineStr"/>
+      <c r="V14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -2202,60 +2391,65 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Cumulus Media</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n">
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>atucker@pcl.com (Alison Tucker, Vice President of Marketing)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>+1 416 201 9995 (Chris Robinson)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="5" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr"/>
-      <c r="O15" s="5" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="5" t="inlineStr"/>
       <c r="Q15" s="5" t="inlineStr"/>
-      <c r="R15" s="4" t="inlineStr">
-        <is>
-          <t>719-593-2700</t>
-        </is>
-      </c>
-      <c r="S15" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
-        </is>
-      </c>
+      <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" s="5" t="inlineStr"/>
+      <c r="T15" s="5" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr"/>
+      <c r="V15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -2263,60 +2457,65 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Ent Credit Union</t>
+          <t>Republic Services</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Credit union</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
+          <t>Waste and recycling</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>jeldridge@republicservices.com (Jennifer Eldridge, Marketing Director)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>+1 480 718 0119 (Jennifer Eldridge)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="4" t="n">
+      <c r="H16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="J16" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>Headquartered in Colorado Springs; about 1,300 staff (Gazette, 2021). Big local sponsor profile.</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>Gazette 2021 (via search; see Fact-check)</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="5" t="inlineStr"/>
-      <c r="N16" s="5" t="inlineStr"/>
-      <c r="O16" s="5" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="5" t="inlineStr"/>
       <c r="Q16" s="5" t="inlineStr"/>
-      <c r="R16" s="4" t="inlineStr">
-        <is>
-          <t>800-525-9623</t>
-        </is>
-      </c>
-      <c r="S16" s="4" t="inlineStr">
-        <is>
-          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
-        </is>
-      </c>
+      <c r="R16" s="5" t="inlineStr"/>
+      <c r="S16" s="5" t="inlineStr"/>
+      <c r="T16" s="5" t="inlineStr"/>
+      <c r="U16" s="4" t="inlineStr"/>
+      <c r="V16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -2324,52 +2523,73 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>McLane Company</t>
+          <t>T. Rowe Price</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Distribution</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
+          <t>Financial services</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>bill_benintende@troweprice.com (Bill Benintende, Vice President of Investments)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>719-278-5600 (Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in))</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="H17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr"/>
-      <c r="M17" s="5" t="inlineStr"/>
-      <c r="N17" s="5" t="inlineStr"/>
-      <c r="O17" s="5" t="inlineStr"/>
+      <c r="K17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Large campus at 2220 Briargate Pkwy, near Chapel Hills Mall. Over 670 staff in 2008 (old figure). Group memberships first, sponsor second.</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>T. Rowe Price locations page and 2008 release (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>To find (HR / benefits for memberships)</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="5" t="inlineStr"/>
       <c r="Q17" s="5" t="inlineStr"/>
-      <c r="R17" s="4" t="inlineStr"/>
-      <c r="S17" s="4" t="inlineStr"/>
+      <c r="R17" s="5" t="inlineStr"/>
+      <c r="S17" s="5" t="inlineStr"/>
+      <c r="T17" s="5" t="inlineStr"/>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>719-278-5600</t>
+        </is>
+      </c>
+      <c r="V17" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -2377,52 +2597,73 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>The Gazette</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Construction</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>michelle.clark@gazette.com (Michelle Clark, Advertising Assistant)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>719-476-1645 (retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G18" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="H18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner: ad space in trade for exposure, or event coverage.</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="5" t="inlineStr"/>
-      <c r="N18" s="5" t="inlineStr"/>
-      <c r="O18" s="5" t="inlineStr"/>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
       <c r="Q18" s="5" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
+      <c r="R18" s="5" t="inlineStr"/>
+      <c r="S18" s="5" t="inlineStr"/>
+      <c r="T18" s="5" t="inlineStr"/>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>719-476-1645</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -2430,52 +2671,73 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Republic Services</t>
+          <t>iHeart Media</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Waste and recycling</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n">
+          <t>Radio</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>kimpiet@iheartmedia.com (Kim Piet, Vice President of Partnerships)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>844-844-4432 (national advertising line (no local number found))</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G19" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="H19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr"/>
-      <c r="M19" s="5" t="inlineStr"/>
-      <c r="N19" s="5" t="inlineStr"/>
-      <c r="O19" s="5" t="inlineStr"/>
+      <c r="O19" s="4" t="inlineStr"/>
       <c r="P19" s="5" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr"/>
-      <c r="R19" s="4" t="inlineStr"/>
-      <c r="S19" s="4" t="inlineStr"/>
+      <c r="R19" s="5" t="inlineStr"/>
+      <c r="S19" s="5" t="inlineStr"/>
+      <c r="T19" s="5" t="inlineStr"/>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>844-844-4432</t>
+        </is>
+      </c>
+      <c r="V19" s="4" t="inlineStr">
+        <is>
+          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -2483,58 +2745,67 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>T. Rowe Price</t>
+          <t>Cheyenne Mountain Resort</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Financial services</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n">
+          <t>Resort</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>719-583-4000 (main line, 3225 Broadmoor Valley Rd)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="4" t="n">
+      <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="J20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>Large campus at 2220 Briargate Pkwy, near Chapel Hills Mall. Over 670 staff in 2008 (old figure). Group memberships first, sponsor second.</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>T. Rowe Price locations page and 2008 release (via search; see Fact-check)</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>To find (HR / benefits for memberships)</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="5" t="inlineStr"/>
-      <c r="N20" s="5" t="inlineStr"/>
-      <c r="O20" s="5" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="4" t="inlineStr">
-        <is>
-          <t>719-278-5600</t>
-        </is>
-      </c>
-      <c r="S20" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" s="5" t="inlineStr"/>
+      <c r="T20" s="5" t="inlineStr"/>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>719-583-4000</t>
+        </is>
+      </c>
+      <c r="V20" s="4" t="inlineStr">
+        <is>
+          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
         </is>
       </c>
     </row>
@@ -2544,60 +2815,61 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>The Gazette</t>
+          <t>Chord Energy</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="n">
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>gilbert.delarosa@chordenergy.com (Gilbert Delarosa, Vice President of Marketing)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner: ad space in trade for exposure, or event coverage.</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr"/>
-      <c r="M21" s="5" t="inlineStr"/>
-      <c r="N21" s="5" t="inlineStr"/>
-      <c r="O21" s="5" t="inlineStr"/>
+      <c r="O21" s="4" t="inlineStr"/>
       <c r="P21" s="5" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr"/>
-      <c r="R21" s="4" t="inlineStr">
-        <is>
-          <t>719-476-1645</t>
-        </is>
-      </c>
-      <c r="S21" s="4" t="inlineStr">
-        <is>
-          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
-        </is>
-      </c>
+      <c r="R21" s="5" t="inlineStr"/>
+      <c r="S21" s="5" t="inlineStr"/>
+      <c r="T21" s="5" t="inlineStr"/>
+      <c r="U21" s="4" t="inlineStr"/>
+      <c r="V21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -2605,60 +2877,65 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>iHeart Media</t>
+          <t>Progressive</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" s="4" t="n">
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>chuck_jarrett@progressive.com (Charles Jarrett, Vice President And Chief Financial Officer)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+1 440 395 2222 (Charles Jarrett)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H22" s="4" t="n">
+      <c r="I22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr"/>
-      <c r="M22" s="5" t="inlineStr"/>
-      <c r="N22" s="5" t="inlineStr"/>
-      <c r="O22" s="5" t="inlineStr"/>
+      <c r="K22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs campus; about 1,500 staff in 2011 (old figure).</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Insurance Journal 2011 (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>To find (HR / benefits for memberships)</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
-      <c r="R22" s="4" t="inlineStr">
-        <is>
-          <t>844-844-4432</t>
-        </is>
-      </c>
-      <c r="S22" s="4" t="inlineStr">
-        <is>
-          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
-        </is>
-      </c>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="5" t="inlineStr"/>
+      <c r="U22" s="4" t="inlineStr"/>
+      <c r="V22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -2666,60 +2943,65 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Altitude Movement</t>
+          <t>USAA</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Fitness / movement</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="n">
+          <t>Insurance / banking</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>jennifer.escobar@usaa.com (Jennifer Escobar, VP of Brand Marketing)</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>+1 916 717 1072 (Roger Wildermuth)</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="4" t="n">
+      <c r="H23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="4" t="n">
+      <c r="I23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr"/>
-      <c r="M23" s="5" t="inlineStr"/>
-      <c r="N23" s="5" t="inlineStr"/>
-      <c r="O23" s="5" t="inlineStr"/>
+      <c r="K23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Large Colorado Springs campus; about 1,800 staff in 2017 (old figure). Military families: Peak’s neighbourhood.</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Area Development 2017 (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>To find (HR / benefits for memberships)</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr"/>
       <c r="P23" s="5" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
-      <c r="R23" s="4" t="inlineStr">
-        <is>
-          <t>719-964-1798</t>
-        </is>
-      </c>
-      <c r="S23" s="4" t="inlineStr">
-        <is>
-          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
-        </is>
-      </c>
+      <c r="R23" s="5" t="inlineStr"/>
+      <c r="S23" s="5" t="inlineStr"/>
+      <c r="T23" s="5" t="inlineStr"/>
+      <c r="U23" s="4" t="inlineStr"/>
+      <c r="V23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -2727,52 +3009,57 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Great Range Bison</t>
+          <t>Climax Molybdenum</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>1</v>
-      </c>
+          <t>Mining</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr"/>
       <c r="F24" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament (name read from its web link; the logo text was unclear).</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr"/>
-      <c r="M24" s="5" t="inlineStr"/>
-      <c r="N24" s="5" t="inlineStr"/>
-      <c r="O24" s="5" t="inlineStr"/>
+      <c r="O24" s="4" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr"/>
       <c r="Q24" s="5" t="inlineStr"/>
-      <c r="R24" s="4" t="inlineStr"/>
-      <c r="S24" s="4" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="5" t="inlineStr"/>
+      <c r="U24" s="4" t="inlineStr"/>
+      <c r="V24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2780,52 +3067,69 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Neon Pig</t>
+          <t>Altitude Movement</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Restaurant</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="n">
+          <t>Fitness / movement</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>719-964-1798 (750 Garden of the Gods Rd #125)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="H25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="J25" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H25" s="4" t="n">
+      <c r="K25" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr"/>
-      <c r="M25" s="5" t="inlineStr"/>
-      <c r="N25" s="5" t="inlineStr"/>
-      <c r="O25" s="5" t="inlineStr"/>
+      <c r="O25" s="4" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
       <c r="Q25" s="5" t="inlineStr"/>
-      <c r="R25" s="4" t="inlineStr"/>
-      <c r="S25" s="4" t="inlineStr"/>
+      <c r="R25" s="5" t="inlineStr"/>
+      <c r="S25" s="5" t="inlineStr"/>
+      <c r="T25" s="5" t="inlineStr"/>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>719-964-1798</t>
+        </is>
+      </c>
+      <c r="V25" s="4" t="inlineStr">
+        <is>
+          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -2833,52 +3137,73 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Progressive</t>
+          <t>Laborjack</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>1</v>
+          <t>Moving / labor</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>jon.emerick@laborjack.com (Jon Emerick, VP of Strategic Alliances)</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>970-690-7709 (Fort Collins office (no Colorado Springs office found))</t>
+        </is>
       </c>
       <c r="F26" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="H26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs campus; about 1,500 staff in 2011 (old figure).</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Insurance Journal 2011 (via search; see Fact-check)</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>To find (HR / benefits for memberships)</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="5" t="inlineStr"/>
-      <c r="N26" s="5" t="inlineStr"/>
-      <c r="O26" s="5" t="inlineStr"/>
+      <c r="I26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr"/>
       <c r="P26" s="5" t="inlineStr"/>
       <c r="Q26" s="5" t="inlineStr"/>
-      <c r="R26" s="4" t="inlineStr"/>
-      <c r="S26" s="4" t="inlineStr"/>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr"/>
+      <c r="T26" s="5" t="inlineStr"/>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>970-690-7709</t>
+        </is>
+      </c>
+      <c r="V26" s="4" t="inlineStr">
+        <is>
+          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -2886,52 +3211,57 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Spartan Barbell</t>
+          <t>Great Range Bison</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="n">
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="G27" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H27" s="4" t="n">
+      <c r="K27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament (name read from its web link; the logo text was unclear).</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr"/>
-      <c r="M27" s="5" t="inlineStr"/>
-      <c r="N27" s="5" t="inlineStr"/>
-      <c r="O27" s="5" t="inlineStr"/>
+      <c r="O27" s="4" t="inlineStr"/>
       <c r="P27" s="5" t="inlineStr"/>
       <c r="Q27" s="5" t="inlineStr"/>
-      <c r="R27" s="4" t="inlineStr"/>
-      <c r="S27" s="4" t="inlineStr"/>
+      <c r="R27" s="5" t="inlineStr"/>
+      <c r="S27" s="5" t="inlineStr"/>
+      <c r="T27" s="5" t="inlineStr"/>
+      <c r="U27" s="4" t="inlineStr"/>
+      <c r="V27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -2939,52 +3269,57 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Spartan Strength Systems</t>
+          <t>Neon Pig</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="n">
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="G28" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H28" s="4" t="n">
+      <c r="K28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr"/>
-      <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr"/>
-      <c r="O28" s="5" t="inlineStr"/>
+      <c r="O28" s="4" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
-      <c r="R28" s="4" t="inlineStr"/>
-      <c r="S28" s="4" t="inlineStr"/>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="5" t="inlineStr"/>
+      <c r="U28" s="4" t="inlineStr"/>
+      <c r="V28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -2992,52 +3327,57 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>USAA</t>
+          <t>Spartan Barbell</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Insurance / banking</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="n">
+          <t>Fitness</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="G29" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G29" s="4" t="n">
+      <c r="J29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>Large Colorado Springs campus; about 1,800 staff in 2017 (old figure). Military families: Peak’s neighbourhood.</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>Area Development 2017 (via search; see Fact-check)</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>To find (HR / benefits for memberships)</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr"/>
-      <c r="M29" s="5" t="inlineStr"/>
-      <c r="N29" s="5" t="inlineStr"/>
-      <c r="O29" s="5" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr"/>
       <c r="P29" s="5" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr"/>
-      <c r="R29" s="4" t="inlineStr"/>
-      <c r="S29" s="4" t="inlineStr"/>
+      <c r="R29" s="5" t="inlineStr"/>
+      <c r="S29" s="5" t="inlineStr"/>
+      <c r="T29" s="5" t="inlineStr"/>
+      <c r="U29" s="4" t="inlineStr"/>
+      <c r="V29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -3045,52 +3385,57 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>KEG1</t>
+          <t>Spartan Strength Systems</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Not checked</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E30" s="4" t="n">
+          <t>Fitness</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr"/>
-      <c r="M30" s="5" t="inlineStr"/>
-      <c r="N30" s="5" t="inlineStr"/>
-      <c r="O30" s="5" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr"/>
       <c r="P30" s="5" t="inlineStr"/>
       <c r="Q30" s="5" t="inlineStr"/>
-      <c r="R30" s="4" t="inlineStr"/>
-      <c r="S30" s="4" t="inlineStr"/>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" s="5" t="inlineStr"/>
+      <c r="T30" s="5" t="inlineStr"/>
+      <c r="U30" s="4" t="inlineStr"/>
+      <c r="V30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -3098,60 +3443,61 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Laborjack</t>
+          <t>Southern Colorado Women’s Chamber of Commerce</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Moving / labor</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="n">
+          <t>Business network</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>lolaw@scwcc.com (Lola Woloch, CEO)</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="I31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Host a member mixer at Peak.</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="5" t="inlineStr"/>
-      <c r="N31" s="5" t="inlineStr"/>
-      <c r="O31" s="5" t="inlineStr"/>
+      <c r="O31" s="4" t="inlineStr"/>
       <c r="P31" s="5" t="inlineStr"/>
       <c r="Q31" s="5" t="inlineStr"/>
-      <c r="R31" s="4" t="inlineStr">
-        <is>
-          <t>970-690-7709</t>
-        </is>
-      </c>
-      <c r="S31" s="4" t="inlineStr">
-        <is>
-          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
-        </is>
-      </c>
+      <c r="R31" s="5" t="inlineStr"/>
+      <c r="S31" s="5" t="inlineStr"/>
+      <c r="T31" s="5" t="inlineStr"/>
+      <c r="U31" s="4" t="inlineStr"/>
+      <c r="V31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -3159,52 +3505,61 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Southern Colorado Women’s Chamber of Commerce</t>
+          <t>Windstar Studios</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="n">
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>elizabeth@windstarstudios.com (Elizabeth Grzelak, President)</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Host a member mixer at Peak.</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="I32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="N32" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr"/>
-      <c r="M32" s="5" t="inlineStr"/>
-      <c r="N32" s="5" t="inlineStr"/>
-      <c r="O32" s="5" t="inlineStr"/>
+      <c r="O32" s="4" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr"/>
       <c r="Q32" s="5" t="inlineStr"/>
-      <c r="R32" s="4" t="inlineStr"/>
-      <c r="S32" s="4" t="inlineStr"/>
+      <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" s="5" t="inlineStr"/>
+      <c r="T32" s="5" t="inlineStr"/>
+      <c r="U32" s="4" t="inlineStr"/>
+      <c r="V32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -3212,7 +3567,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Windstar Studios</t>
+          <t>KEG1</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -3220,44 +3575,49 @@
           <t>Not checked</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G33" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="I33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr"/>
-      <c r="M33" s="5" t="inlineStr"/>
-      <c r="N33" s="5" t="inlineStr"/>
-      <c r="O33" s="5" t="inlineStr"/>
+      <c r="O33" s="4" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
       <c r="Q33" s="5" t="inlineStr"/>
-      <c r="R33" s="4" t="inlineStr"/>
-      <c r="S33" s="4" t="inlineStr"/>
+      <c r="R33" s="5" t="inlineStr"/>
+      <c r="S33" s="5" t="inlineStr"/>
+      <c r="T33" s="5" t="inlineStr"/>
+      <c r="U33" s="4" t="inlineStr"/>
+      <c r="V33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3265,52 +3625,61 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>BCA</t>
+          <t>Dwire Earthmoving, LLC</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Not checked</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="n">
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>jeff@dwirex.com (Jeff Dwire, Owner)</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="H34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="M34" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr"/>
-      <c r="M34" s="5" t="inlineStr"/>
-      <c r="N34" s="5" t="inlineStr"/>
-      <c r="O34" s="5" t="inlineStr"/>
+      <c r="O34" s="4" t="inlineStr"/>
       <c r="P34" s="5" t="inlineStr"/>
       <c r="Q34" s="5" t="inlineStr"/>
-      <c r="R34" s="4" t="inlineStr"/>
-      <c r="S34" s="4" t="inlineStr"/>
+      <c r="R34" s="5" t="inlineStr"/>
+      <c r="S34" s="5" t="inlineStr"/>
+      <c r="T34" s="5" t="inlineStr"/>
+      <c r="U34" s="4" t="inlineStr"/>
+      <c r="V34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -3318,52 +3687,69 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Baker and King</t>
+          <t>Hispanic Chamber of Commerce</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Not checked</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="n">
+          <t>Business network</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>719-231-5353 (Colorado Springs Hispanic Chamber)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="H35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="I35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Host a member mixer at Peak.</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr"/>
-      <c r="M35" s="5" t="inlineStr"/>
-      <c r="N35" s="5" t="inlineStr"/>
-      <c r="O35" s="5" t="inlineStr"/>
+      <c r="O35" s="4" t="inlineStr"/>
       <c r="P35" s="5" t="inlineStr"/>
       <c r="Q35" s="5" t="inlineStr"/>
-      <c r="R35" s="4" t="inlineStr"/>
-      <c r="S35" s="4" t="inlineStr"/>
+      <c r="R35" s="5" t="inlineStr"/>
+      <c r="S35" s="5" t="inlineStr"/>
+      <c r="T35" s="5" t="inlineStr"/>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>719-231-5353</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3371,52 +3757,57 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Dwire Earthmoving, LLC</t>
+          <t>BCA</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Construction</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="n">
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G36" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="M36" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr"/>
-      <c r="M36" s="5" t="inlineStr"/>
-      <c r="N36" s="5" t="inlineStr"/>
-      <c r="O36" s="5" t="inlineStr"/>
+      <c r="O36" s="4" t="inlineStr"/>
       <c r="P36" s="5" t="inlineStr"/>
       <c r="Q36" s="5" t="inlineStr"/>
-      <c r="R36" s="4" t="inlineStr"/>
-      <c r="S36" s="4" t="inlineStr"/>
+      <c r="R36" s="5" t="inlineStr"/>
+      <c r="S36" s="5" t="inlineStr"/>
+      <c r="T36" s="5" t="inlineStr"/>
+      <c r="U36" s="4" t="inlineStr"/>
+      <c r="V36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3424,60 +3815,57 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Hispanic Chamber of Commerce</t>
+          <t>Baker and King</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="n">
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G37" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Host a member mixer at Peak.</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="I37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr"/>
-      <c r="M37" s="5" t="inlineStr"/>
-      <c r="N37" s="5" t="inlineStr"/>
-      <c r="O37" s="5" t="inlineStr"/>
+      <c r="O37" s="4" t="inlineStr"/>
       <c r="P37" s="5" t="inlineStr"/>
       <c r="Q37" s="5" t="inlineStr"/>
-      <c r="R37" s="4" t="inlineStr">
-        <is>
-          <t>719-231-5353</t>
-        </is>
-      </c>
-      <c r="S37" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
-        </is>
-      </c>
+      <c r="R37" s="5" t="inlineStr"/>
+      <c r="S37" s="5" t="inlineStr"/>
+      <c r="T37" s="5" t="inlineStr"/>
+      <c r="U37" s="4" t="inlineStr"/>
+      <c r="V37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -3493,44 +3881,49 @@
           <t>Retail</t>
         </is>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G38" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="I38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Family audience.</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="M38" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr"/>
-      <c r="M38" s="5" t="inlineStr"/>
-      <c r="N38" s="5" t="inlineStr"/>
-      <c r="O38" s="5" t="inlineStr"/>
+      <c r="O38" s="4" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr"/>
       <c r="Q38" s="5" t="inlineStr"/>
-      <c r="R38" s="4" t="inlineStr"/>
-      <c r="S38" s="4" t="inlineStr"/>
+      <c r="R38" s="5" t="inlineStr"/>
+      <c r="S38" s="5" t="inlineStr"/>
+      <c r="T38" s="5" t="inlineStr"/>
+      <c r="U38" s="4" t="inlineStr"/>
+      <c r="V38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -3546,44 +3939,49 @@
           <t>Not checked</t>
         </is>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G39" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="I39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="M39" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L39" s="4" t="inlineStr"/>
-      <c r="M39" s="5" t="inlineStr"/>
-      <c r="N39" s="5" t="inlineStr"/>
-      <c r="O39" s="5" t="inlineStr"/>
+      <c r="O39" s="4" t="inlineStr"/>
       <c r="P39" s="5" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr"/>
-      <c r="R39" s="4" t="inlineStr"/>
-      <c r="S39" s="4" t="inlineStr"/>
+      <c r="R39" s="5" t="inlineStr"/>
+      <c r="S39" s="5" t="inlineStr"/>
+      <c r="T39" s="5" t="inlineStr"/>
+      <c r="U39" s="4" t="inlineStr"/>
+      <c r="V39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -3599,49 +3997,54 @@
           <t>Consulting</t>
         </is>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G40" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="I40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="M40" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr">
+      <c r="N40" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="L40" s="4" t="inlineStr"/>
-      <c r="M40" s="5" t="inlineStr"/>
-      <c r="N40" s="5" t="inlineStr"/>
-      <c r="O40" s="5" t="inlineStr"/>
+      <c r="O40" s="4" t="inlineStr"/>
       <c r="P40" s="5" t="inlineStr"/>
       <c r="Q40" s="5" t="inlineStr"/>
-      <c r="R40" s="4" t="inlineStr"/>
-      <c r="S40" s="4" t="inlineStr"/>
+      <c r="R40" s="5" t="inlineStr"/>
+      <c r="S40" s="5" t="inlineStr"/>
+      <c r="T40" s="5" t="inlineStr"/>
+      <c r="U40" s="4" t="inlineStr"/>
+      <c r="V40" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S40"/>
+  <autoFilter ref="A1:V40"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,Emailed,Called,Tour booked,Toured,Proposal sent,Signed,Not now,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5315,7 +5718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J197"/>
+  <dimension ref="A1:J199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12405,31 +12808,27 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Peak Pelvic Health (local)</t>
+          <t>Kaiser Permanente</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>Mallory Willis</t>
-        </is>
-      </c>
-      <c r="C178" s="4" t="inlineStr"/>
+          <t>Colorado community sponsorships</t>
+        </is>
+      </c>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t>Sponsorship inbox (rules exclude advertising)</t>
+        </is>
+      </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>mallory@peakpelvichealthco.com</t>
-        </is>
-      </c>
-      <c r="E178" s="4" t="n">
-        <v>99</v>
-      </c>
-      <c r="F178" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G178" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
+          <t>communityco@kp.org</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="n"/>
+      <c r="F178" s="4" t="n"/>
+      <c r="G178" s="4" t="inlineStr"/>
       <c r="H178" s="4" t="inlineStr"/>
       <c r="I178" s="4" t="inlineStr">
         <is>
@@ -12441,12 +12840,12 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Peak Pelvic Health (local)</t>
+          <t>Colorado Springs Chamber &amp; EDC</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>General inbox</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
@@ -12456,54 +12855,50 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>info@peakpelvichealthco.com</t>
-        </is>
-      </c>
-      <c r="E179" s="4" t="n">
-        <v>77</v>
-      </c>
-      <c r="F179" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G179" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
+          <t>info@cscedc.com</t>
+        </is>
+      </c>
+      <c r="E179" s="4" t="n"/>
+      <c r="F179" s="4" t="n"/>
+      <c r="G179" s="4" t="inlineStr"/>
       <c r="H179" s="4" t="inlineStr"/>
-      <c r="I179" s="4" t="inlineStr"/>
-      <c r="J179" s="4" t="inlineStr"/>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>Ask for first</t>
+        </is>
+      </c>
+      <c r="J179" s="4" t="inlineStr">
+        <is>
+          <t>719-471-8183</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>ABC Family Chiropractic (local)</t>
+          <t>Peak Pelvic Health (local)</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
-        </is>
-      </c>
-      <c r="C180" s="4" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
+          <t>Mallory Willis</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr"/>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>info@abcfamilychiropractic.com</t>
+          <t>mallory@peakpelvichealthco.com</t>
         </is>
       </c>
       <c r="E180" s="4" t="n">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="F180" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G180" s="4" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="H180" s="4" t="inlineStr"/>
@@ -12517,73 +12912,77 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Therapy Center North (local)</t>
+          <t>Peak Pelvic Health (local)</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>Hailey Burns</t>
+          <t>general inbox</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Occupational Therapy Manager</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>haileyb@cstherapycenter.com</t>
+          <t>info@peakpelvichealthco.com</t>
         </is>
       </c>
       <c r="E181" s="4" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F181" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G181" s="4" t="inlineStr">
         <is>
-          <t>2025-03-26</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="H181" s="4" t="inlineStr"/>
-      <c r="I181" s="4" t="inlineStr">
-        <is>
-          <t>Ask for first</t>
-        </is>
-      </c>
+      <c r="I181" s="4" t="inlineStr"/>
       <c r="J181" s="4" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Therapy Center North (local)</t>
+          <t>ABC Family Chiropractic (local)</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>Craig Peterson</t>
-        </is>
-      </c>
-      <c r="C182" s="4" t="inlineStr"/>
+          <t>general inbox</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>craigp@cstherapycenter.com</t>
+          <t>info@abcfamilychiropractic.com</t>
         </is>
       </c>
       <c r="E182" s="4" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="F182" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G182" s="4" t="inlineStr">
         <is>
-          <t>2025-10-31</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="H182" s="4" t="inlineStr"/>
-      <c r="I182" s="4" t="inlineStr"/>
+      <c r="I182" s="4" t="inlineStr">
+        <is>
+          <t>Ask for first</t>
+        </is>
+      </c>
       <c r="J182" s="4" t="inlineStr"/>
     </row>
     <row r="183">
@@ -12594,32 +12993,36 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>Hailey Burns</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>Occupational Therapy Manager</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>info@cstherapycenter.com</t>
+          <t>haileyb@cstherapycenter.com</t>
         </is>
       </c>
       <c r="E183" s="4" t="n">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F183" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G183" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2025-03-26</t>
         </is>
       </c>
       <c r="H183" s="4" t="inlineStr"/>
-      <c r="I183" s="4" t="inlineStr"/>
+      <c r="I183" s="4" t="inlineStr">
+        <is>
+          <t>Ask for first</t>
+        </is>
+      </c>
       <c r="J183" s="4" t="inlineStr"/>
     </row>
     <row r="184">
@@ -12630,28 +13033,24 @@
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
-        </is>
-      </c>
-      <c r="C184" s="4" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
+          <t>Craig Peterson</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr"/>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>office@cstherapycenter.com</t>
+          <t>craigp@cstherapycenter.com</t>
         </is>
       </c>
       <c r="E184" s="4" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="F184" s="4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G184" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2025-10-31</t>
         </is>
       </c>
       <c r="H184" s="4" t="inlineStr"/>
@@ -12661,113 +13060,105 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>Revolution Rehabilitation, P.C. (local)</t>
+          <t>Colorado Springs Therapy Center North (local)</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>Kamber Arbini</t>
+          <t>general inbox</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>kamber@revrehab.com</t>
+          <t>info@cstherapycenter.com</t>
         </is>
       </c>
       <c r="E185" s="4" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F185" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G185" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H185" s="4" t="inlineStr"/>
-      <c r="I185" s="4" t="inlineStr">
-        <is>
-          <t>Ask for first</t>
-        </is>
-      </c>
+      <c r="I185" s="4" t="inlineStr"/>
       <c r="J185" s="4" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Wholistic Healing Experiences (local)</t>
+          <t>Colorado Springs Therapy Center North (local)</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>Dawn Ramsden</t>
+          <t>general inbox</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>dawn@wholistichealingexperiences.com</t>
+          <t>office@cstherapycenter.com</t>
         </is>
       </c>
       <c r="E186" s="4" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="F186" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G186" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="H186" s="4" t="inlineStr"/>
-      <c r="I186" s="4" t="inlineStr">
-        <is>
-          <t>Ask for first</t>
-        </is>
-      </c>
+      <c r="I186" s="4" t="inlineStr"/>
       <c r="J186" s="4" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>Manual Edge Physiotherapist (local)</t>
+          <t>Revolution Rehabilitation, P.C. (local)</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>Kamber Arbini</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>referrals@manualedge.com</t>
+          <t>kamber@revrehab.com</t>
         </is>
       </c>
       <c r="E187" s="4" t="n">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="F187" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G187" s="4" t="inlineStr">
         <is>
-          <t>2025-10-10</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="H187" s="4" t="inlineStr"/>
@@ -12781,69 +13172,73 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>Manual Edge Physiotherapist (local)</t>
+          <t>Wholistic Healing Experiences (local)</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>Dawn Ramsden</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>letstalk@manualedge.com</t>
+          <t>dawn@wholistichealingexperiences.com</t>
         </is>
       </c>
       <c r="E188" s="4" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="F188" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G188" s="4" t="inlineStr">
         <is>
-          <t>2025-10-12</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H188" s="4" t="inlineStr"/>
-      <c r="I188" s="4" t="inlineStr"/>
+      <c r="I188" s="4" t="inlineStr">
+        <is>
+          <t>Ask for first</t>
+        </is>
+      </c>
       <c r="J188" s="4" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>Lakeside Auto Brokers (local)</t>
+          <t>Manual Edge Physiotherapist (local)</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>Tiffany Beacham</t>
+          <t>general inbox</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
         <is>
-          <t>tiffanyb@lakesideautobrokers.com</t>
+          <t>referrals@manualedge.com</t>
         </is>
       </c>
       <c r="E189" s="4" t="n">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="F189" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G189" s="4" t="inlineStr">
         <is>
-          <t>2025-08-16</t>
+          <t>2025-10-10</t>
         </is>
       </c>
       <c r="H189" s="4" t="inlineStr"/>
@@ -12857,69 +13252,69 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>The Faricy Boys Chrysler Jeep (local)</t>
+          <t>Manual Edge Physiotherapist (local)</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>Paul Faricy</t>
-        </is>
-      </c>
-      <c r="C190" s="4" t="inlineStr"/>
+          <t>general inbox</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
       <c r="D190" s="4" t="inlineStr">
         <is>
-          <t>pfaricy@faricy.com</t>
+          <t>letstalk@manualedge.com</t>
         </is>
       </c>
       <c r="E190" s="4" t="n">
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="F190" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G190" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2025-10-12</t>
         </is>
       </c>
       <c r="H190" s="4" t="inlineStr"/>
-      <c r="I190" s="4" t="inlineStr">
-        <is>
-          <t>Ask for first</t>
-        </is>
-      </c>
+      <c r="I190" s="4" t="inlineStr"/>
       <c r="J190" s="4" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>Keller Williams Clients' Choice Realty (local)</t>
+          <t>Lakeside Auto Brokers (local)</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>Tiffany Beacham</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>frontdesk@ourkwteam.com</t>
+          <t>tiffanyb@lakesideautobrokers.com</t>
         </is>
       </c>
       <c r="E191" s="4" t="n">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="F191" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G191" s="4" t="inlineStr">
         <is>
-          <t>2025-10-21</t>
+          <t>2025-08-16</t>
         </is>
       </c>
       <c r="H191" s="4" t="inlineStr"/>
@@ -12933,33 +13328,29 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>More Than Your Money, Inc. (local)</t>
+          <t>The Faricy Boys Chrysler Jeep (local)</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>Jane Young</t>
-        </is>
-      </c>
-      <c r="C192" s="4" t="inlineStr">
-        <is>
-          <t>President</t>
-        </is>
-      </c>
+          <t>Paul Faricy</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr"/>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>jane@morethanyourmoney.com</t>
+          <t>pfaricy@faricy.com</t>
         </is>
       </c>
       <c r="E192" s="4" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="F192" s="4" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="G192" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="H192" s="4" t="inlineStr"/>
@@ -12973,33 +13364,33 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>Foundation Professionals of Colorado (local)</t>
+          <t>Keller Williams Clients' Choice Realty (local)</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>Angie Martin</t>
+          <t>general inbox</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>General Manager</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>angie.martin@foundationprosofco.com</t>
+          <t>frontdesk@ourkwteam.com</t>
         </is>
       </c>
       <c r="E193" s="4" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="F193" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G193" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="H193" s="4" t="inlineStr"/>
@@ -13013,33 +13404,33 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>Whole Living Pilattes (local)</t>
+          <t>More Than Your Money, Inc. (local)</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>Jane Young</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>President</t>
         </is>
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>info@wholelivingpilates.com</t>
+          <t>jane@morethanyourmoney.com</t>
         </is>
       </c>
       <c r="E194" s="4" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F194" s="4" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="G194" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="H194" s="4" t="inlineStr"/>
@@ -13053,29 +13444,29 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>Homestead Roofing, Inc (local)</t>
+          <t>Foundation Professionals of Colorado (local)</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>Tracy Bookman</t>
+          <t>Angie Martin</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Customer Service</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>tracy@homesteadroofingcolorado.com</t>
+          <t>angie.martin@foundationprosofco.com</t>
         </is>
       </c>
       <c r="E195" s="4" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F195" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G195" s="4" t="inlineStr">
         <is>
@@ -13093,7 +13484,7 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>Homestead Roofing, Inc (local)</t>
+          <t>Whole Living Pilattes (local)</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
@@ -13108,54 +13499,58 @@
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>info@homesteadroofingcolorado.com</t>
+          <t>info@wholelivingpilates.com</t>
         </is>
       </c>
       <c r="E196" s="4" t="n">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="F196" s="4" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G196" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="H196" s="4" t="inlineStr"/>
-      <c r="I196" s="4" t="inlineStr"/>
+      <c r="I196" s="4" t="inlineStr">
+        <is>
+          <t>Ask for first</t>
+        </is>
+      </c>
       <c r="J196" s="4" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Klaus Roofing (local)</t>
+          <t>Homestead Roofing, Inc (local)</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>general inbox</t>
+          <t>Tracy Bookman</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>Customer Service</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>info@klausroofingcolorado.com</t>
+          <t>tracy@homesteadroofingcolorado.com</t>
         </is>
       </c>
       <c r="E197" s="4" t="n">
         <v>99</v>
       </c>
       <c r="F197" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G197" s="4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="H197" s="4" t="inlineStr"/>
@@ -13166,8 +13561,84 @@
       </c>
       <c r="J197" s="4" t="inlineStr"/>
     </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>Homestead Roofing, Inc (local)</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>general inbox</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>info@homesteadroofingcolorado.com</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="F198" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G198" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H198" s="4" t="inlineStr"/>
+      <c r="I198" s="4" t="inlineStr"/>
+      <c r="J198" s="4" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>Klaus Roofing (local)</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>general inbox</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D199" s="4" t="inlineStr">
+        <is>
+          <t>info@klausroofingcolorado.com</t>
+        </is>
+      </c>
+      <c r="E199" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G199" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H199" s="4" t="inlineStr"/>
+      <c r="I199" s="4" t="inlineStr">
+        <is>
+          <t>Ask for first</t>
+        </is>
+      </c>
+      <c r="J199" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J197"/>
+  <autoFilter ref="A1:J199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Peak leads grouped: phone and email, then phone only, then email only, then neither; score within each (Matthew 2026-10-21); sheet, brief and live desk
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
+++ b/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
@@ -1324,7 +1324,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Order points (score + email + phone)</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
@@ -1461,25 +1461,31 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Kaiser Permanente</t>
+          <t>UCHealth (Memorial Hospital; Memorial North)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Health insurer / care</t>
+          <t>Hospital system</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>communityco@kp.org (Colorado community sponsorships, Sponsorship inbox (rules exclude advertising))</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="n">
-        <v>9</v>
+          <t>todd.seip@uchealth.org (Todd Seip, Director Of Public Relations)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>+1 719 584 4499 (Todd Seip)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>3</v>
@@ -1488,27 +1494,31 @@
         <v>3</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>Paid sponsor of the Colorado Chamber’s 2024 pickleball tournament (Pickle Hour and awards) at the Broadmoor.</t>
+          <t>No. 4 employer in El Paso County (7,050 staff, 2024). Gives through community grants (southern Colorado grants announced in UCHealth news).</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>https://epc-assets.elpasoco.com/wp-content/uploads/sites/2/2024-ACFR-FINAL-reduced-size.pdf ; https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>To find (statewide marketing; check for a Colorado Springs community contact)</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr"/>
+          <t>Community and government affairs, southern Colorado (the senior director is named in UCHealth news releases). Also an employee-membership target (see Employers).</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
+        </is>
+      </c>
       <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr"/>
@@ -1523,60 +1533,62 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>UCHealth (Memorial Hospital; Memorial North)</t>
+          <t>Alpine Bank</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Hospital system</t>
+          <t>Bank</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>todd.seip@uchealth.org (Todd Seip, Director Of Public Relations)</t>
+          <t>alansandberg@alpinebank.com (Alan Sandberg, Director Of Marketing)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>+1 719 584 4499 (Todd Seip)</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>9</v>
+          <t>719-421-7600 (Colorado Springs branch, 90 S Cascade Ave, Ste 100)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>No. 4 employer in El Paso County (7,050 staff, 2024). Gives through community grants (southern Colorado grants announced in UCHealth news).</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>https://epc-assets.elpasoco.com/wp-content/uploads/sites/2/2024-ACFR-FINAL-reduced-size.pdf ; https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>Community and government affairs, southern Colorado (the senior director is named in UCHealth news releases). Also an employee-membership target (see Employers).</t>
+          <t>Front Range sponsorship request form (to its Denver office; asks 60 days ahead). The form may be dated: confirm the current contact first.</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
+          <t>https://www.alpinebank.com/custom/fi/alpinebank/fb/disclosure/Sponsorship_Request_Form_Front-Range.pdf</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr"/>
@@ -1584,8 +1596,16 @@
       <c r="R3" s="5" t="inlineStr"/>
       <c r="S3" s="5" t="inlineStr"/>
       <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
-      <c r="V3" s="4" t="inlineStr"/>
+      <c r="U3" s="4" t="inlineStr">
+        <is>
+          <t>719-421-7600</t>
+        </is>
+      </c>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs branch, 90 S Cascade Ave, Ste 100 · https://www.alpinebank.com/locations/colorado-springs.html</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -1593,7 +1613,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Alpine Bank</t>
+          <t>BOK Financial</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1603,16 +1623,18 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>alansandberg@alpinebank.com (Alan Sandberg, Director Of Marketing)</t>
+          <t>ggerst@bokf.com (Gilbert Gerst, Senior Vice President Community Development)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>719-421-7600 (Colorado Springs branch, 90 S Cascade Ave, Ste 100)</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>8</v>
+          <t>303-863-4270 (Colorado commercial banking (no Colorado Springs office listed))</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G4" s="4" t="n">
         <v>6</v>
@@ -1631,7 +1653,7 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -1641,14 +1663,10 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>Front Range sponsorship request form (to its Denver office; asks 60 days ahead). The form may be dated: confirm the current contact first.</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>https://www.alpinebank.com/custom/fi/alpinebank/fb/disclosure/Sponsorship_Request_Form_Front-Range.pdf</t>
-        </is>
-      </c>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
       <c r="R4" s="5" t="inlineStr"/>
@@ -1656,12 +1674,12 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>719-421-7600</t>
+          <t>303-863-4270</t>
         </is>
       </c>
       <c r="V4" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs branch, 90 S Cascade Ave, Ste 100 · https://www.alpinebank.com/locations/colorado-springs.html</t>
+          <t>Colorado commercial banking (no Colorado Springs office listed) · https://bokfinancial.com/location-and-contact-us/additional-contact-information/CO</t>
         </is>
       </c>
     </row>
@@ -1671,26 +1689,28 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>BOK Financial</t>
+          <t>Molson Coors</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Bank</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>ggerst@bokf.com (Gilbert Gerst, Senior Vice President Community Development)</t>
+          <t>meghan.means@molsoncoors.com (Meghan Means, Marketing Director)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>303-863-4270 (Colorado commercial banking (no Colorado Springs office listed))</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>8</v>
+          <t>303-279-6565 (head office, Golden)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G5" s="4" t="n">
         <v>6</v>
@@ -1709,12 +1729,12 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -1730,12 +1750,12 @@
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>303-863-4270</t>
+          <t>303-279-6565</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t>Colorado commercial banking (no Colorado Springs office listed) · https://bokfinancial.com/location-and-contact-us/additional-contact-information/CO</t>
+          <t>head office, Golden · SEC EDGAR filing, business phone</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1765,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Molson Coors</t>
+          <t>Coca-Cola</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1755,19 +1775,21 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>meghan.means@molsoncoors.com (Meghan Means, Marketing Director)</t>
+          <t>apopescu@swirecc.com (Andrei Popescu, Marketing Director)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>303-279-6565 (head office, Golden)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>8</v>
+          <t>719-257-5745 (Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>1</v>
@@ -1776,19 +1798,19 @@
         <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Also a pouring-rights deal for Peak’s snack bar, if Peak has one.</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -1804,12 +1826,12 @@
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>303-279-6565</t>
+          <t>719-257-5745</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t>head office, Golden · SEC EDGAR filing, business phone</t>
+          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
         </is>
       </c>
     </row>
@@ -1819,31 +1841,37 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>OrangeTheory</t>
+          <t>Colorado Media Group</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>memberservices@orangetheory.com (General inbox)</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="n">
-        <v>7</v>
+          <t>dhobbs@coloradomediagroup.com (Dirk Hobbs, Division Manager)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>719-330-7448 (publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs))</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>2</v>
@@ -1853,7 +1881,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner, as above.</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -1863,7 +1891,7 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>To find (franchise: the local owner decides)</t>
+          <t>To find</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr"/>
@@ -1872,8 +1900,16 @@
       <c r="R7" s="5" t="inlineStr"/>
       <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
-      <c r="U7" s="4" t="inlineStr"/>
-      <c r="V7" s="4" t="inlineStr"/>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>719-330-7448</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs) · https://www.visitcos.com/directory/colorado-media-group-real-estate/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -1881,26 +1917,28 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Coca-Cola</t>
+          <t>Colorado Springs Chamber &amp; EDC</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Beverage</t>
+          <t>Business network</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>apopescu@swirecc.com (Andrei Popescu, Marketing Director)</t>
+          <t>info@cscedc.com (General inbox)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>719-257-5745 (Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs)</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>7</v>
+          <t>719-471-8183 (main line)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G8" s="4" t="n">
         <v>5</v>
@@ -1909,17 +1947,17 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Also a pouring-rights deal for Peak’s snack bar, if Peak has one.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Introductions to members and a venue for a member event at Peak.</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -1940,12 +1978,12 @@
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>719-257-5745</t>
+          <t>719-471-8183</t>
         </is>
       </c>
       <c r="V8" s="4" t="inlineStr">
         <is>
-          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
+          <t>main line; email info@cscedc.com · https://coloradospringschamberedc.com/contact/</t>
         </is>
       </c>
     </row>
@@ -1955,26 +1993,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Colorado Media Group</t>
+          <t>Concept Restaurants</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Restaurant group</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>dhobbs@coloradomediagroup.com (Dirk Hobbs, Division Manager)</t>
+          <t>erin@conceptrestaurants.com (Erin Copeland, Vice President of Marketing)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>719-330-7448 (publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs))</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>7</v>
+          <t>719-635-3536 (MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A))</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G9" s="4" t="n">
         <v>5</v>
@@ -1993,7 +2033,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner, as above.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -2014,12 +2054,12 @@
       <c r="T9" s="5" t="inlineStr"/>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>719-330-7448</t>
+          <t>719-635-3536</t>
         </is>
       </c>
       <c r="V9" s="4" t="inlineStr">
         <is>
-          <t>publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs) · https://www.visitcos.com/directory/colorado-media-group-real-estate/</t>
+          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
         </is>
       </c>
     </row>
@@ -2029,26 +2069,28 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Chamber &amp; EDC</t>
+          <t>Cumulus Media</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>info@cscedc.com (General inbox)</t>
+          <t>james.robinson@cumulus.com (James Robinson, Vice President, Marketing)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>719-471-8183 (main line)</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>7</v>
+          <t>719-593-2700 (Colorado Springs stations, 6805 Corporate Dr #130)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G10" s="4" t="n">
         <v>5</v>
@@ -2067,7 +2109,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Introductions to members and a venue for a member event at Peak.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -2088,12 +2130,12 @@
       <c r="T10" s="5" t="inlineStr"/>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>719-471-8183</t>
+          <t>719-593-2700</t>
         </is>
       </c>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>main line; email info@cscedc.com · https://coloradospringschamberedc.com/contact/</t>
+          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
         </is>
       </c>
     </row>
@@ -2103,26 +2145,28 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Concept Restaurants</t>
+          <t>Ent Credit Union</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Restaurant group</t>
+          <t>Credit union</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>erin@conceptrestaurants.com (Erin Copeland, Vice President of Marketing)</t>
+          <t>kutermoehlen@ent.com (Kelly Utermoehlen, Director of Internal Communications)</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>719-635-3536 (MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A))</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>7</v>
+          <t>800-525-9623 (main line)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G11" s="4" t="n">
         <v>5</v>
@@ -2131,22 +2175,22 @@
         <v>1</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+          <t>Headquartered in Colorado Springs; about 1,300 staff (Gazette, 2021). Big local sponsor profile.</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Gazette 2021 (via search; see Fact-check)</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -2162,12 +2206,12 @@
       <c r="T11" s="5" t="inlineStr"/>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>719-635-3536</t>
+          <t>800-525-9623</t>
         </is>
       </c>
       <c r="V11" s="4" t="inlineStr">
         <is>
-          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
+          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
         </is>
       </c>
     </row>
@@ -2177,35 +2221,37 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Cumulus Media</t>
+          <t>McLane Company</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Distribution</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>james.robinson@cumulus.com (James Robinson, Vice President, Marketing)</t>
+          <t>tom.sicola@mclaneco.com (Tom Sicola, Vp Of Marketing)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>719-593-2700 (Colorado Springs stations, 6805 Corporate Dr #130)</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>7</v>
+          <t>+1 254 742 3637 (Tom Sicola)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
@@ -2215,12 +2261,12 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -2234,16 +2280,8 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr"/>
       <c r="T12" s="5" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>719-593-2700</t>
-        </is>
-      </c>
-      <c r="V12" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
-        </is>
-      </c>
+      <c r="U12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2251,50 +2289,52 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ent Credit Union</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Credit union</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>kutermoehlen@ent.com (Kelly Utermoehlen, Director of Internal Communications)</t>
+          <t>atucker@pcl.com (Alison Tucker, Vice President of Marketing)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>800-525-9623 (main line)</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>7</v>
+          <t>+1 416 201 9995 (Chris Robinson)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G13" s="4" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Headquartered in Colorado Springs; about 1,300 staff (Gazette, 2021). Big local sponsor profile.</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Gazette 2021 (via search; see Fact-check)</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -2308,16 +2348,8 @@
       <c r="R13" s="5" t="inlineStr"/>
       <c r="S13" s="5" t="inlineStr"/>
       <c r="T13" s="5" t="inlineStr"/>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>800-525-9623</t>
-        </is>
-      </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
-        </is>
-      </c>
+      <c r="U13" s="4" t="inlineStr"/>
+      <c r="V13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -2325,26 +2357,28 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>McLane Company</t>
+          <t>Republic Services</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Distribution</t>
+          <t>Waste and recycling</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>tom.sicola@mclaneco.com (Tom Sicola, Vp Of Marketing)</t>
+          <t>jeldridge@republicservices.com (Jennifer Eldridge, Marketing Director)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>+1 254 742 3637 (Tom Sicola)</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>7</v>
+          <t>+1 480 718 0119 (Jennifer Eldridge)</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G14" s="4" t="n">
         <v>5</v>
@@ -2363,12 +2397,12 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -2391,55 +2425,57 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>T. Rowe Price</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Financial services</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>atucker@pcl.com (Alison Tucker, Vice President of Marketing)</t>
+          <t>bill_benintende@troweprice.com (Bill Benintende, Vice President of Investments)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>+1 416 201 9995 (Chris Robinson)</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>7</v>
+          <t>719-278-5600 (Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in))</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G15" s="4" t="n">
         <v>5</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+          <t>Large campus at 2220 Briargate Pkwy, near Chapel Hills Mall. Over 670 staff in 2008 (old figure). Group memberships first, sponsor second.</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>T. Rowe Price locations page and 2008 release (via search; see Fact-check)</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
+          <t>To find (HR / benefits for memberships)</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr"/>
@@ -2448,8 +2484,16 @@
       <c r="R15" s="5" t="inlineStr"/>
       <c r="S15" s="5" t="inlineStr"/>
       <c r="T15" s="5" t="inlineStr"/>
-      <c r="U15" s="4" t="inlineStr"/>
-      <c r="V15" s="4" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>719-278-5600</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -2457,35 +2501,37 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Republic Services</t>
+          <t>The Gazette</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Waste and recycling</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>jeldridge@republicservices.com (Jennifer Eldridge, Marketing Director)</t>
+          <t>michelle.clark@gazette.com (Michelle Clark, Advertising Assistant)</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>+1 480 718 0119 (Jennifer Eldridge)</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>7</v>
+          <t>719-476-1645 (retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G16" s="4" t="n">
         <v>5</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>2</v>
@@ -2495,7 +2541,7 @@
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner: ad space in trade for exposure, or event coverage.</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -2514,8 +2560,16 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr"/>
       <c r="T16" s="5" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr"/>
-      <c r="V16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>719-476-1645</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="inlineStr">
+        <is>
+          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -2523,26 +2577,28 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>T. Rowe Price</t>
+          <t>iHeart Media</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Financial services</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>bill_benintende@troweprice.com (Bill Benintende, Vice President of Investments)</t>
+          <t>kimpiet@iheartmedia.com (Kim Piet, Vice President of Partnerships)</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>719-278-5600 (Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in))</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>7</v>
+          <t>844-844-4432 (national advertising line (no local number found))</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G17" s="4" t="n">
         <v>5</v>
@@ -2551,27 +2607,27 @@
         <v>1</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Large campus at 2220 Briargate Pkwy, near Chapel Hills Mall. Over 670 staff in 2008 (old figure). Group memberships first, sponsor second.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>T. Rowe Price locations page and 2008 release (via search; see Fact-check)</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>To find (HR / benefits for memberships)</t>
+          <t>To find</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr"/>
@@ -2582,12 +2638,12 @@
       <c r="T17" s="5" t="inlineStr"/>
       <c r="U17" s="4" t="inlineStr">
         <is>
-          <t>719-278-5600</t>
+          <t>844-844-4432</t>
         </is>
       </c>
       <c r="V17" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
         </is>
       </c>
     </row>
@@ -2597,55 +2653,57 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>The Gazette</t>
+          <t>Progressive</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>michelle.clark@gazette.com (Michelle Clark, Advertising Assistant)</t>
+          <t>chuck_jarrett@progressive.com (Charles Jarrett, Vice President And Chief Financial Officer)</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>719-476-1645 (retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave)</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>7</v>
+          <t>+1 440 395 2222 (Charles Jarrett)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G18" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner: ad space in trade for exposure, or event coverage.</t>
+          <t>Colorado Springs campus; about 1,500 staff in 2011 (old figure).</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Insurance Journal 2011 (via search; see Fact-check)</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
+          <t>To find (HR / benefits for memberships)</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr"/>
@@ -2654,16 +2712,8 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr">
-        <is>
-          <t>719-476-1645</t>
-        </is>
-      </c>
-      <c r="V18" s="4" t="inlineStr">
-        <is>
-          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
-        </is>
-      </c>
+      <c r="U18" s="4" t="inlineStr"/>
+      <c r="V18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -2671,55 +2721,57 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>iHeart Media</t>
+          <t>USAA</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Insurance / banking</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>kimpiet@iheartmedia.com (Kim Piet, Vice President of Partnerships)</t>
+          <t>jennifer.escobar@usaa.com (Jennifer Escobar, VP of Brand Marketing)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>844-844-4432 (national advertising line (no local number found))</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>7</v>
+          <t>+1 916 717 1072 (Roger Wildermuth)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
+          <t>Large Colorado Springs campus; about 1,800 staff in 2017 (old figure). Military families: Peak’s neighbourhood.</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Area Development 2017 (via search; see Fact-check)</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
+          <t>To find (HR / benefits for memberships)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr"/>
@@ -2728,16 +2780,8 @@
       <c r="R19" s="5" t="inlineStr"/>
       <c r="S19" s="5" t="inlineStr"/>
       <c r="T19" s="5" t="inlineStr"/>
-      <c r="U19" s="4" t="inlineStr">
-        <is>
-          <t>844-844-4432</t>
-        </is>
-      </c>
-      <c r="V19" s="4" t="inlineStr">
-        <is>
-          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
-        </is>
-      </c>
+      <c r="U19" s="4" t="inlineStr"/>
+      <c r="V19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -2745,31 +2789,37 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Cheyenne Mountain Resort</t>
+          <t>Laborjack</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Resort</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
+          <t>Moving / labor</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>jon.emerick@laborjack.com (Jon Emerick, VP of Strategic Alliances)</t>
+        </is>
+      </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>719-583-4000 (main line, 3225 Broadmoor Valley Rd)</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>6</v>
+          <t>970-690-7709 (Fort Collins office (no Colorado Springs office found))</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Phone and email</t>
+        </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>2</v>
@@ -2779,7 +2829,7 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
@@ -2800,12 +2850,12 @@
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>719-583-4000</t>
+          <t>970-690-7709</t>
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr">
         <is>
-          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
+          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
         </is>
       </c>
     </row>
@@ -2815,22 +2865,24 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Chord Energy</t>
+          <t>Cheyenne Mountain Resort</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>gilbert.delarosa@chordenergy.com (Gilbert Delarosa, Vice President of Marketing)</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="n">
-        <v>6</v>
+          <t>Resort</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>719-583-4000 (main line, 3225 Broadmoor Valley Rd)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Phone only</t>
+        </is>
       </c>
       <c r="G21" s="4" t="n">
         <v>5</v>
@@ -2849,12 +2901,12 @@
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -2868,8 +2920,16 @@
       <c r="R21" s="5" t="inlineStr"/>
       <c r="S21" s="5" t="inlineStr"/>
       <c r="T21" s="5" t="inlineStr"/>
-      <c r="U21" s="4" t="inlineStr"/>
-      <c r="V21" s="4" t="inlineStr"/>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>719-583-4000</t>
+        </is>
+      </c>
+      <c r="V21" s="4" t="inlineStr">
+        <is>
+          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -2877,55 +2937,53 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Progressive</t>
+          <t>Altitude Movement</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>chuck_jarrett@progressive.com (Charles Jarrett, Vice President And Chief Financial Officer)</t>
-        </is>
-      </c>
+          <t>Fitness / movement</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>+1 440 395 2222 (Charles Jarrett)</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>6</v>
+          <t>719-964-1798 (750 Garden of the Gods Rd #125)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Phone only</t>
+        </is>
       </c>
       <c r="G22" s="4" t="n">
         <v>4</v>
       </c>
       <c r="H22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="J22" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs campus; about 1,500 staff in 2011 (old figure).</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>Insurance Journal 2011 (via search; see Fact-check)</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>To find (HR / benefits for memberships)</t>
+          <t>To find</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr"/>
@@ -2934,8 +2992,16 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
-      <c r="U22" s="4" t="inlineStr"/>
-      <c r="V22" s="4" t="inlineStr"/>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>719-964-1798</t>
+        </is>
+      </c>
+      <c r="V22" s="4" t="inlineStr">
+        <is>
+          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -2943,55 +3009,53 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>USAA</t>
+          <t>Hispanic Chamber of Commerce</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Insurance / banking</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>jennifer.escobar@usaa.com (Jennifer Escobar, VP of Brand Marketing)</t>
-        </is>
-      </c>
+          <t>Business network</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>+1 916 717 1072 (Roger Wildermuth)</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>6</v>
+          <t>719-231-5353 (Colorado Springs Hispanic Chamber)</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Phone only</t>
+        </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I23" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="J23" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Large Colorado Springs campus; about 1,800 staff in 2017 (old figure). Military families: Peak’s neighbourhood.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Host a member mixer at Peak.</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Area Development 2017 (via search; see Fact-check)</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>To find (HR / benefits for memberships)</t>
+          <t>To find</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr"/>
@@ -3000,8 +3064,16 @@
       <c r="R23" s="5" t="inlineStr"/>
       <c r="S23" s="5" t="inlineStr"/>
       <c r="T23" s="5" t="inlineStr"/>
-      <c r="U23" s="4" t="inlineStr"/>
-      <c r="V23" s="4" t="inlineStr"/>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>719-231-5353</t>
+        </is>
+      </c>
+      <c r="V23" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -3009,24 +3081,30 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Climax Molybdenum</t>
+          <t>Kaiser Permanente</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Mining</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
+          <t>Health insurer / care</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>communityco@kp.org (Colorado community sponsorships, Sponsorship inbox (rules exclude advertising))</t>
+        </is>
+      </c>
       <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="n">
-        <v>5</v>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Email only</t>
+        </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I24" s="4" t="n">
         <v>3</v>
@@ -3039,7 +3117,7 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+          <t>Paid sponsor of the Colorado Chamber’s 2024 pickleball tournament (Pickle Hour and awards) at the Broadmoor.</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -3049,7 +3127,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
+          <t>To find (statewide marketing; check for a Colorado Springs community contact)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr"/>
@@ -3067,41 +3145,43 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Altitude Movement</t>
+          <t>OrangeTheory</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Fitness / movement</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>719-964-1798 (750 Garden of the Gods Rd #125)</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>5</v>
+          <t>Fitness</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>memberservices@orangetheory.com (General inbox)</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Email only</t>
+        </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>1</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -3111,7 +3191,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
+          <t>To find (franchise: the local owner decides)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr"/>
@@ -3120,16 +3200,8 @@
       <c r="R25" s="5" t="inlineStr"/>
       <c r="S25" s="5" t="inlineStr"/>
       <c r="T25" s="5" t="inlineStr"/>
-      <c r="U25" s="4" t="inlineStr">
-        <is>
-          <t>719-964-1798</t>
-        </is>
-      </c>
-      <c r="V25" s="4" t="inlineStr">
-        <is>
-          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
-        </is>
-      </c>
+      <c r="U25" s="4" t="inlineStr"/>
+      <c r="V25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -3137,35 +3209,33 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Laborjack</t>
+          <t>Chord Energy</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Moving / labor</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>jon.emerick@laborjack.com (Jon Emerick, VP of Strategic Alliances)</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>970-690-7709 (Fort Collins office (no Colorado Springs office found))</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n">
+          <t>gilbert.delarosa@chordenergy.com (Gilbert Delarosa, Vice President of Marketing)</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Email only</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="H26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J26" s="4" t="n">
         <v>2</v>
@@ -3175,12 +3245,12 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -3194,16 +3264,8 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr"/>
-      <c r="U26" s="4" t="inlineStr">
-        <is>
-          <t>970-690-7709</t>
-        </is>
-      </c>
-      <c r="V26" s="4" t="inlineStr">
-        <is>
-          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
-        </is>
-      </c>
+      <c r="U26" s="4" t="inlineStr"/>
+      <c r="V26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -3211,24 +3273,30 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Great Range Bison</t>
+          <t>Southern Colorado Women’s Chamber of Commerce</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr"/>
+          <t>Business network</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>lolaw@scwcc.com (Lola Woloch, CEO)</t>
+        </is>
+      </c>
       <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="n">
-        <v>4</v>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Email only</t>
+        </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" s="4" t="n">
         <v>1</v>
@@ -3241,12 +3309,12 @@
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament (name read from its web link; the logo text was unclear).</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Host a member mixer at Peak.</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -3269,24 +3337,30 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Neon Pig</t>
+          <t>Windstar Studios</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Restaurant</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>elizabeth@windstarstudios.com (Elizabeth Grzelak, President)</t>
+        </is>
+      </c>
       <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="n">
-        <v>4</v>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Email only</t>
+        </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" s="4" t="n">
         <v>1</v>
@@ -3299,7 +3373,7 @@
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
@@ -3327,24 +3401,30 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Spartan Barbell</t>
+          <t>Dwire Earthmoving, LLC</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>jeff@dwirex.com (Jeff Dwire, Owner)</t>
+        </is>
+      </c>
       <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="n">
-        <v>4</v>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Email only</t>
+        </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I29" s="4" t="n">
         <v>1</v>
@@ -3385,42 +3465,44 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Spartan Strength Systems</t>
+          <t>Climax Molybdenum</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
+          <t>Mining</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="n">
-        <v>4</v>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="I30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="K30" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
@@ -3443,28 +3525,26 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Southern Colorado Women’s Chamber of Commerce</t>
+          <t>Great Range Bison</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>lolaw@scwcc.com (Lola Woloch, CEO)</t>
-        </is>
-      </c>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="n">
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G31" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="H31" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>1</v>
@@ -3477,12 +3557,12 @@
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Host a member mixer at Peak.</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament (name read from its web link; the logo text was unclear).</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
@@ -3505,28 +3585,26 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Windstar Studios</t>
+          <t>Neon Pig</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Not checked</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>elizabeth@windstarstudios.com (Elizabeth Grzelak, President)</t>
-        </is>
-      </c>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="n">
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G32" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="H32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="4" t="n">
         <v>1</v>
@@ -3539,7 +3617,7 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
@@ -3567,37 +3645,39 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>KEG1</t>
+          <t>Spartan Barbell</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Not checked</t>
+          <t>Fitness</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="n">
-        <v>3</v>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="J33" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K33" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
@@ -3625,28 +3705,26 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Dwire Earthmoving, LLC</t>
+          <t>Spartan Strength Systems</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Construction</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>jeff@dwirex.com (Jeff Dwire, Owner)</t>
-        </is>
-      </c>
+          <t>Fitness</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="4" t="n">
-        <v>3</v>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G34" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H34" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="H34" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="I34" s="4" t="n">
         <v>1</v>
@@ -3687,25 +3765,23 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Hispanic Chamber of Commerce</t>
+          <t>KEG1</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>719-231-5353 (Colorado Springs Hispanic Chamber)</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="n">
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="H35" s="4" t="n">
         <v>0</v>
@@ -3714,14 +3790,14 @@
         <v>1</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K35" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Host a member mixer at Peak.</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
@@ -3740,16 +3816,8 @@
       <c r="R35" s="5" t="inlineStr"/>
       <c r="S35" s="5" t="inlineStr"/>
       <c r="T35" s="5" t="inlineStr"/>
-      <c r="U35" s="4" t="inlineStr">
-        <is>
-          <t>719-231-5353</t>
-        </is>
-      </c>
-      <c r="V35" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
-        </is>
-      </c>
+      <c r="U35" s="4" t="inlineStr"/>
+      <c r="V35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3767,8 +3835,10 @@
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="n">
-        <v>2</v>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G36" s="4" t="n">
         <v>2</v>
@@ -3825,8 +3895,10 @@
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="n">
-        <v>2</v>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G37" s="4" t="n">
         <v>2</v>
@@ -3883,8 +3955,10 @@
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr"/>
-      <c r="F38" s="4" t="n">
-        <v>2</v>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G38" s="4" t="n">
         <v>2</v>
@@ -3941,8 +4015,10 @@
       </c>
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="n">
-        <v>2</v>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G39" s="4" t="n">
         <v>2</v>
@@ -3999,8 +4075,10 @@
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="4" t="n">
-        <v>2</v>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Neither yet</t>
+        </is>
       </c>
       <c r="G40" s="4" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Peak leads ordered by who the phone reaches (Matthew 2026-10-21: "prioritize the ones that lead to a good person"; "make those 3 changes")
data/call-quality.json: each number judged: direct to a good person (UCHealth, Alpine, Coca-Cola/Swire, McLane, Republic), a small
organisation's main line (Chamber, Hispanic Chamber, Colorado Media Group, Altitude Movement, Cumulus), a front desk to ask by name
(Molson Coors, Ent, T. Rowe Price, Laborjack, Cheyenne Mountain), or weak/wrong (BOK, PCL, Progressive, USAA off the best-phone spot;
Concept, Gazette, iHeart: email first). Each lead gets a "how to call" line (direct to X / front desk: ask for X, title); media companies:
pitch a trade, not their ad sales. Sheet (Best phone, How to call, Group), brief and live desk (highlighted call line, "Best contact
first" order). desk 34/34 before upload.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
+++ b/matthew/peak-pickleball-sponsorship/Peak-Sponsor-Leads-2026-10.xlsx
@@ -21,7 +21,7 @@
     <sheet name="Pitch and tour invite" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$V$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsor leads'!$A$1:$W$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Renewals (Peak sponsors)'!$A$1:$G$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Employers 400+'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'What others charge'!$A$1:$H$13</definedName>
@@ -1316,31 +1316,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V40"/>
+  <dimension ref="A1:W40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="58" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="44" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="26" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="40" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1371,85 +1372,90 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
+          <t>How to call</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Score /9</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Fit /3</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Money /3</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Sponsors sport /2</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Near Peak /1</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Why they fit</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Route in</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Route link</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Contact (name, role)</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Email / phone</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Next step / date</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Main / local phone</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>Phone source</t>
         </is>
@@ -1476,56 +1482,61 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>+1 719 584 4499 (Todd Seip)</t>
+          <t>719-584-4499</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="n">
+          <t>Direct to Todd Seip, Director of Public Relations (local 719 number)</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Direct to a good person</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="I2" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J2" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>No. 4 employer in El Paso County (7,050 staff, 2024). Gives through community grants (southern Colorado grants announced in UCHealth news).</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>https://epc-assets.elpasoco.com/wp-content/uploads/sites/2/2024-ACFR-FINAL-reduced-size.pdf ; https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Community and government affairs, southern Colorado (the senior director is named in UCHealth news releases). Also an employee-membership target (see Employers).</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>https://www.aol.com/articles/uchealth-awards-218-000-grants-014454931.html</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr"/>
       <c r="T2" s="5" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
+      <c r="U2" s="5" t="inlineStr"/>
       <c r="V2" s="4" t="inlineStr"/>
+      <c r="W2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1548,60 +1559,65 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>719-421-7600 (Colorado Springs branch, 90 S Cascade Ave, Ste 100)</t>
+          <t>970-384-3216</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n">
+          <t>Direct to Alan Sandberg, Director of Marketing (head office area code). Colorado Springs branch: 719-421-7600</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Direct to a good person</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Front Range sponsorship request form (to its Denver office; asks 60 days ahead). The form may be dated: confirm the current contact first.</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>https://www.alpinebank.com/custom/fi/alpinebank/fb/disclosure/Sponsorship_Request_Form_Front-Range.pdf</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
       <c r="R3" s="5" t="inlineStr"/>
       <c r="S3" s="5" t="inlineStr"/>
       <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr">
         <is>
           <t>719-421-7600</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
+      <c r="W3" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs branch, 90 S Cascade Ave, Ste 100 · https://www.alpinebank.com/locations/colorado-springs.html</t>
         </is>
@@ -1613,73 +1629,78 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>BOK Financial</t>
+          <t>Coca-Cola</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Bank</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>ggerst@bokf.com (Gilbert Gerst, Senior Vice President Community Development)</t>
+          <t>apopescu@swirecc.com (Andrei Popescu, Marketing Director)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>303-863-4270 (Colorado commercial banking (no Colorado Springs office listed))</t>
+          <t>801-816-5714</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>6</v>
+          <t>Direct to Michele McKillip, SVP Corporate Affairs (corporate affairs often handles sponsorships). Colorado Springs distribution center: 719-257-5745</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Direct to a good person</t>
+        </is>
       </c>
       <c r="H4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="K4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Also a pouring-rights deal for Peak’s snack bar, if Peak has one.</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr"/>
       <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>303-863-4270</t>
-        </is>
-      </c>
+      <c r="U4" s="5" t="inlineStr"/>
       <c r="V4" s="4" t="inlineStr">
         <is>
-          <t>Colorado commercial banking (no Colorado Springs office listed) · https://bokfinancial.com/location-and-contact-us/additional-contact-information/CO</t>
+          <t>719-257-5745</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
         </is>
       </c>
     </row>
@@ -1689,75 +1710,72 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Molson Coors</t>
+          <t>McLane Company</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Beverage</t>
+          <t>Distribution</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>meghan.means@molsoncoors.com (Meghan Means, Marketing Director)</t>
+          <t>tom.sicola@mclaneco.com (Tom Sicola, Vp Of Marketing)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>303-279-6565 (head office, Golden)</t>
+          <t>254-742-3637</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>6</v>
+          <t>Direct to Tom Sicola, VP of Marketing (Texas head office)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Direct to a good person</t>
+        </is>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
-        </is>
-      </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="5" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
       <c r="S5" s="5" t="inlineStr"/>
       <c r="T5" s="5" t="inlineStr"/>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>303-279-6565</t>
-        </is>
-      </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>head office, Golden · SEC EDGAR filing, business phone</t>
-        </is>
-      </c>
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="4" t="inlineStr"/>
+      <c r="W5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -1765,75 +1783,72 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Coca-Cola</t>
+          <t>Republic Services</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Beverage</t>
+          <t>Waste and recycling</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>apopescu@swirecc.com (Andrei Popescu, Marketing Director)</t>
+          <t>jeldridge@republicservices.com (Jennifer Eldridge, Marketing Director)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>719-257-5745 (Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs)</t>
+          <t>480-718-0119</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="n">
+          <t>Direct to Jennifer Eldridge, Marketing Director (Phoenix head office)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Direct to a good person</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="K6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Also a pouring-rights deal for Peak’s snack bar, if Peak has one.</t>
-        </is>
-      </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
       <c r="Q6" s="5" t="inlineStr"/>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr"/>
       <c r="T6" s="5" t="inlineStr"/>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>719-257-5745</t>
-        </is>
-      </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>Swire Coca-Cola distribution center, 1935 Cygnet Heights, Colorado Springs · https://www.swirecc.com/Colorado</t>
-        </is>
-      </c>
+      <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -1856,56 +1871,61 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>719-330-7448 (publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs))</t>
+          <t>719-330-7448</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="n">
+          <t>Main line (North magazine); ask for Dirk Hobbs, Division Manager. Pitch a media trade, not a cash buy</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Main line, small organisation</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner, as above.</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="5" t="inlineStr"/>
+      <c r="P7" s="4" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr"/>
       <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
-      <c r="U7" s="4" t="inlineStr">
+      <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7" s="4" t="inlineStr">
         <is>
           <t>719-330-7448</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>publisher of North magazine, 13395 Voyager Pkwy, Ste 130 (north Colorado Springs) · https://www.visitcos.com/directory/colorado-media-group-real-estate/</t>
         </is>
@@ -1932,56 +1952,61 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>719-471-8183 (main line)</t>
+          <t>719-471-8183</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n">
+          <t>Main line; small staff. Ask who handles events and member partnerships</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Main line, small organisation</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Introductions to members and a venue for a member event at Peak.</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr"/>
       <c r="T8" s="5" t="inlineStr"/>
-      <c r="U8" s="4" t="inlineStr">
+      <c r="U8" s="5" t="inlineStr"/>
+      <c r="V8" s="4" t="inlineStr">
         <is>
           <t>719-471-8183</t>
         </is>
       </c>
-      <c r="V8" s="4" t="inlineStr">
+      <c r="W8" s="4" t="inlineStr">
         <is>
           <t>main line; email info@cscedc.com · https://coloradospringschamberedc.com/contact/</t>
         </is>
@@ -1993,73 +2018,78 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Concept Restaurants</t>
+          <t>Cumulus Media</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Restaurant group</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>erin@conceptrestaurants.com (Erin Copeland, Vice President of Marketing)</t>
+          <t>james.robinson@cumulus.com (James Robinson, Vice President, Marketing)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>719-635-3536 (MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A))</t>
+          <t>719-593-2700</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="n">
+          <t>Colorado Springs stations; ask for Scott Jones, VP/Market Manager. Pitch a media trade (their airtime for Peak exposure), not ad sales</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Main line, small organisation</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="5" t="inlineStr"/>
+      <c r="P9" s="4" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
       <c r="R9" s="5" t="inlineStr"/>
       <c r="S9" s="5" t="inlineStr"/>
       <c r="T9" s="5" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>719-635-3536</t>
-        </is>
-      </c>
+      <c r="U9" s="5" t="inlineStr"/>
       <c r="V9" s="4" t="inlineStr">
         <is>
-          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
+          <t>719-593-2700</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
         </is>
       </c>
     </row>
@@ -2069,73 +2099,74 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Cumulus Media</t>
+          <t>Altitude Movement</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>james.robinson@cumulus.com (James Robinson, Vice President, Marketing)</t>
-        </is>
-      </c>
+          <t>Fitness / movement</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>719-593-2700 (Colorado Springs stations, 6805 Corporate Dr #130)</t>
+          <t>719-964-1798</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>5</v>
+          <t>Main line; small gym, ask for the owner</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Main line, small organisation</t>
+        </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
-        </is>
-      </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="5" t="inlineStr"/>
+      <c r="P10" s="4" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr"/>
       <c r="T10" s="5" t="inlineStr"/>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>719-593-2700</t>
-        </is>
-      </c>
+      <c r="U10" s="5" t="inlineStr"/>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs stations, 6805 Corporate Dr #130; VP/Market Manager Scott Jones (Cumulus releases) · BBB listings for the Colorado Springs stations</t>
+          <t>719-964-1798</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
         </is>
       </c>
     </row>
@@ -2145,73 +2176,74 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ent Credit Union</t>
+          <t>Hispanic Chamber of Commerce</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Credit union</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>kutermoehlen@ent.com (Kelly Utermoehlen, Director of Internal Communications)</t>
-        </is>
-      </c>
+          <t>Business network</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>800-525-9623 (main line)</t>
+          <t>719-231-5353</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>5</v>
+          <t>Main line; ask for Joe Aldaz, President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Main line, small organisation</t>
+        </is>
       </c>
       <c r="H11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Headquartered in Colorado Springs; about 1,300 staff (Gazette, 2021). Big local sponsor profile.</t>
-        </is>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>Gazette 2021 (via search; see Fact-check)</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Host a member mixer at Peak.</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr"/>
-      <c r="P11" s="5" t="inlineStr"/>
+      <c r="P11" s="4" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>800-525-9623</t>
-        </is>
-      </c>
+      <c r="U11" s="5" t="inlineStr"/>
       <c r="V11" s="4" t="inlineStr">
         <is>
-          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
+          <t>719-231-5353</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
         </is>
       </c>
     </row>
@@ -2221,67 +2253,80 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>McLane Company</t>
+          <t>Molson Coors</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Distribution</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>tom.sicola@mclaneco.com (Tom Sicola, Vp Of Marketing)</t>
+          <t>meghan.means@molsoncoors.com (Meghan Means, Marketing Director)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>+1 254 742 3637 (Tom Sicola)</t>
+          <t>303-279-6565</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>5</v>
+          <t>Head office front desk: ask for Meghan Means, Marketing Director</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Front desk: ask by name</t>
+        </is>
       </c>
       <c r="H12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
-      </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament at the Broadmoor.</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="5" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr"/>
       <c r="T12" s="5" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="inlineStr"/>
+      <c r="U12" s="5" t="inlineStr"/>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>303-279-6565</t>
+        </is>
+      </c>
+      <c r="W12" s="4" t="inlineStr">
+        <is>
+          <t>head office, Golden · SEC EDGAR filing, business phone</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2289,67 +2334,80 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>Ent Credit Union</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Credit union</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>atucker@pcl.com (Alison Tucker, Vice President of Marketing)</t>
+          <t>kutermoehlen@ent.com (Kelly Utermoehlen, Director of Internal Communications)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>+1 416 201 9995 (Chris Robinson)</t>
+          <t>800-525-9623</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="n">
+          <t>Front desk: ask for marketing (Kelly Utermoehlen, Director of Internal Communications, is the closest name found)</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Front desk: ask by name</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
+      <c r="L13" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>Headquartered in Colorado Springs; about 1,300 staff (Gazette, 2021). Big local sponsor profile.</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
+          <t>Gazette 2021 (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="5" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
       <c r="R13" s="5" t="inlineStr"/>
       <c r="S13" s="5" t="inlineStr"/>
       <c r="T13" s="5" t="inlineStr"/>
-      <c r="U13" s="4" t="inlineStr"/>
-      <c r="V13" s="4" t="inlineStr"/>
+      <c r="U13" s="5" t="inlineStr"/>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>800-525-9623</t>
+        </is>
+      </c>
+      <c r="W13" s="4" t="inlineStr">
+        <is>
+          <t>main line; ask for marketing · https://www.ent.com/contact-us</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -2357,67 +2415,80 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Republic Services</t>
+          <t>T. Rowe Price</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Waste and recycling</t>
+          <t>Financial services</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>jeldridge@republicservices.com (Jennifer Eldridge, Marketing Director)</t>
+          <t>bill_benintende@troweprice.com (Bill Benintende, Vice President of Investments)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>+1 480 718 0119 (Jennifer Eldridge)</t>
+          <t>719-278-5600</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="n">
+          <t>Colorado Springs campus switchboard: ask who handles local community or employee programs (lead with group memberships)</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Front desk: ask by name</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
+      <c r="L14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Large campus at 2220 Briargate Pkwy, near Chapel Hills Mall. Over 670 staff in 2008 (old figure). Group memberships first, sponsor second.</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="5" t="inlineStr"/>
+          <t>T. Rowe Price locations page and 2008 release (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>To find (HR / benefits for memberships)</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr"/>
       <c r="Q14" s="5" t="inlineStr"/>
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr"/>
       <c r="T14" s="5" t="inlineStr"/>
-      <c r="U14" s="4" t="inlineStr"/>
-      <c r="V14" s="4" t="inlineStr"/>
+      <c r="U14" s="5" t="inlineStr"/>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>719-278-5600</t>
+        </is>
+      </c>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -2425,73 +2496,78 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>T. Rowe Price</t>
+          <t>Laborjack</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Financial services</t>
+          <t>Moving / labor</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>bill_benintende@troweprice.com (Bill Benintende, Vice President of Investments)</t>
+          <t>jon.emerick@laborjack.com (Jon Emerick, VP of Strategic Alliances)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>719-278-5600 (Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in))</t>
+          <t>970-690-7709</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>5</v>
+          <t>Fort Collins office: ask for Jon Emerick, VP of Strategic Alliances</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Front desk: ask by name</t>
+        </is>
       </c>
       <c r="H15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I15" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J15" s="4" t="n">
+      <c r="K15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Large campus at 2220 Briargate Pkwy, near Chapel Hills Mall. Over 670 staff in 2008 (old figure). Group memberships first, sponsor second.</t>
-        </is>
-      </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>T. Rowe Price locations page and 2008 release (via search; see Fact-check)</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>To find (HR / benefits for memberships)</t>
-        </is>
-      </c>
-      <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="5" t="inlineStr"/>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="5" t="inlineStr"/>
       <c r="R15" s="5" t="inlineStr"/>
       <c r="S15" s="5" t="inlineStr"/>
       <c r="T15" s="5" t="inlineStr"/>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>719-278-5600</t>
-        </is>
-      </c>
+      <c r="U15" s="5" t="inlineStr"/>
       <c r="V15" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs campus, 2220 Briargate Pkwy (operations center, no walk-in) · https://troweprice.com/corporate/us/en/locations.html</t>
+          <t>970-690-7709</t>
+        </is>
+      </c>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
         </is>
       </c>
     </row>
@@ -2501,73 +2577,74 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>The Gazette</t>
+          <t>Cheyenne Mountain Resort</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>michelle.clark@gazette.com (Michelle Clark, Advertising Assistant)</t>
-        </is>
-      </c>
+          <t>Resort</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>719-476-1645 (retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave)</t>
+          <t>719-583-4000</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="n">
+          <t>Front desk: ask for sales or marketing (check first whether they run their own pickleball courts)</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Front desk: ask by name</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H16" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner: ad space in trade for exposure, or event coverage.</t>
-        </is>
-      </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="5" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="5" t="inlineStr"/>
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr"/>
       <c r="T16" s="5" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr">
-        <is>
-          <t>719-476-1645</t>
-        </is>
-      </c>
+      <c r="U16" s="5" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr">
         <is>
-          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
+          <t>719-583-4000</t>
+        </is>
+      </c>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
         </is>
       </c>
     </row>
@@ -2577,75 +2654,64 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>iHeart Media</t>
+          <t>Kaiser Permanente</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>Health insurer / care</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>kimpiet@iheartmedia.com (Kim Piet, Vice President of Partnerships)</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>844-844-4432 (national advertising line (no local number found))</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>5</v>
+          <t>communityco@kp.org (Colorado community sponsorships, Sponsorship inbox (rules exclude advertising))</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K17" s="4" t="n">
+      <c r="L17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
-        </is>
-      </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Paid sponsor of the Colorado Chamber’s 2024 pickleball tournament (Pickle Hour and awards) at the Broadmoor.</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="O17" s="4" t="inlineStr"/>
-      <c r="P17" s="5" t="inlineStr"/>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>To find (statewide marketing; check for a Colorado Springs community contact)</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="5" t="inlineStr"/>
       <c r="R17" s="5" t="inlineStr"/>
       <c r="S17" s="5" t="inlineStr"/>
       <c r="T17" s="5" t="inlineStr"/>
-      <c r="U17" s="4" t="inlineStr">
-        <is>
-          <t>844-844-4432</t>
-        </is>
-      </c>
-      <c r="V17" s="4" t="inlineStr">
-        <is>
-          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
-        </is>
-      </c>
+      <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -2653,67 +2719,76 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Progressive</t>
+          <t>BOK Financial</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Bank</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>chuck_jarrett@progressive.com (Charles Jarrett, Vice President And Chief Financial Officer)</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>+1 440 395 2222 (Charles Jarrett)</t>
-        </is>
-      </c>
+          <t>ggerst@bokf.com (Gilbert Gerst, Senior Vice President Community Development)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>4</v>
+          <t>No good number: the Colorado line (303-863-4270) is commercial banking. Email Gilbert Gerst, SVP Community Development</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="J18" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="K18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs campus; about 1,500 staff in 2011 (old figure).</t>
-        </is>
-      </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Insurance Journal 2011 (via search; see Fact-check)</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>To find (HR / benefits for memberships)</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="5" t="inlineStr"/>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="5" t="inlineStr"/>
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="inlineStr"/>
+      <c r="U18" s="5" t="inlineStr"/>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>303-863-4270</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>Colorado commercial banking (no Colorado Springs office listed) · https://bokfinancial.com/location-and-contact-us/additional-contact-information/CO</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -2721,67 +2796,64 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>USAA</t>
+          <t>OrangeTheory</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Insurance / banking</t>
+          <t>Fitness</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>jennifer.escobar@usaa.com (Jennifer Escobar, VP of Brand Marketing)</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>+1 916 717 1072 (Roger Wildermuth)</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>4</v>
+          <t>memberservices@orangetheory.com (General inbox)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H19" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I19" s="4" t="n">
         <v>3</v>
       </c>
       <c r="J19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Large Colorado Springs campus; about 1,800 staff in 2017 (old figure). Military families: Peak’s neighbourhood.</t>
-        </is>
-      </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>Area Development 2017 (via search; see Fact-check)</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>To find (HR / benefits for memberships)</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="5" t="inlineStr"/>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>To find (franchise: the local owner decides)</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr"/>
       <c r="R19" s="5" t="inlineStr"/>
       <c r="S19" s="5" t="inlineStr"/>
       <c r="T19" s="5" t="inlineStr"/>
-      <c r="U19" s="4" t="inlineStr"/>
+      <c r="U19" s="5" t="inlineStr"/>
       <c r="V19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -2789,75 +2861,64 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Laborjack</t>
+          <t>Chord Energy</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Moving / labor</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>jon.emerick@laborjack.com (Jon Emerick, VP of Strategic Alliances)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>970-690-7709 (Fort Collins office (no Colorado Springs office found))</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Phone and email</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="n">
+          <t>gilbert.delarosa@chordenergy.com (Gilbert Delarosa, Vice President of Marketing)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="K20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
-        </is>
-      </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="5" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr">
-        <is>
-          <t>970-690-7709</t>
-        </is>
-      </c>
-      <c r="V20" s="4" t="inlineStr">
-        <is>
-          <t>Fort Collins office (no Colorado Springs office found) · moving-company directory listings</t>
-        </is>
-      </c>
+      <c r="U20" s="5" t="inlineStr"/>
+      <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -2865,69 +2926,78 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Cheyenne Mountain Resort</t>
+          <t>Concept Restaurants</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Resort</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr"/>
+          <t>Restaurant group</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>erin@conceptrestaurants.com (Erin Copeland, Vice President of Marketing)</t>
+        </is>
+      </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>719-583-4000 (main line, 3225 Broadmoor Valley Rd)</t>
+          <t>719-635-3536</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Phone only</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="n">
+          <t>Only a restaurant front desk (MacKenzie's Chop House). Email Erin Copeland, VP of Marketing, first</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H21" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I21" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Check first whether it runs its own courts (could be a competitor).</t>
-        </is>
-      </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="5" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr"/>
       <c r="R21" s="5" t="inlineStr"/>
       <c r="S21" s="5" t="inlineStr"/>
       <c r="T21" s="5" t="inlineStr"/>
-      <c r="U21" s="4" t="inlineStr">
-        <is>
-          <t>719-583-4000</t>
-        </is>
-      </c>
+      <c r="U21" s="5" t="inlineStr"/>
       <c r="V21" s="4" t="inlineStr">
         <is>
-          <t>main line, 3225 Broadmoor Valley Rd · hotel and venue listings (consistent)</t>
+          <t>719-635-3536</t>
+        </is>
+      </c>
+      <c r="W21" s="4" t="inlineStr">
+        <is>
+          <t>MacKenzie's Chop House, 128 S Tejon (named as a Concept restaurant in a Gazette Q&amp;A); no corporate line found · Chamber directory and restaurant listings</t>
         </is>
       </c>
     </row>
@@ -2937,71 +3007,68 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Altitude Movement</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Fitness / movement</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>719-964-1798 (750 Garden of the Gods Rd #125)</t>
-        </is>
-      </c>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>atucker@pcl.com (Alison Tucker, Vice President of Marketing)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Phone only</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>4</v>
+          <t>No good number (the one found is a labour-relations director in Toronto). Email Alison Tucker, VP of Marketing</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H22" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="I22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="4" t="n">
+      <c r="L22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
-        </is>
-      </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
+          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="5" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>719-964-1798</t>
-        </is>
-      </c>
-      <c r="V22" s="4" t="inlineStr">
-        <is>
-          <t>750 Garden of the Gods Rd #125 · Macaroni Kid Colorado Springs directory</t>
-        </is>
-      </c>
+      <c r="U22" s="5" t="inlineStr"/>
+      <c r="V22" s="4" t="inlineStr"/>
+      <c r="W22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -3009,69 +3076,78 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Hispanic Chamber of Commerce</t>
+          <t>The Gazette</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Business network</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>michelle.clark@gazette.com (Michelle Clark, Advertising Assistant)</t>
+        </is>
+      </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>719-231-5353 (Colorado Springs Hispanic Chamber)</t>
+          <t>719-632-5511</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Phone only</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>2</v>
+          <t>Main line; the ad lines sell ads, they don't buy. Ask for marketing or promotions and pitch a media trade</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I23" s="4" t="n">
         <v>1</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Host a member mixer at Peak.</t>
-        </is>
-      </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
+          <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport. Media partner: ad space in trade for exposure, or event coverage.</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="5" t="inlineStr"/>
+      <c r="P23" s="4" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
       <c r="R23" s="5" t="inlineStr"/>
       <c r="S23" s="5" t="inlineStr"/>
       <c r="T23" s="5" t="inlineStr"/>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>719-231-5353</t>
-        </is>
-      </c>
+      <c r="U23" s="5" t="inlineStr"/>
       <c r="V23" s="4" t="inlineStr">
         <is>
-          <t>Colorado Springs Hispanic Chamber; President &amp; CEO Joe Aldaz · chamber directory listings (consistent number)</t>
+          <t>719-476-1645</t>
+        </is>
+      </c>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>retail advertising (main line 719-632-5511), 30 E Pikes Peak Ave · https://gazette.com/contact-us/</t>
         </is>
       </c>
     </row>
@@ -3081,63 +3157,80 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Kaiser Permanente</t>
+          <t>iHeart Media</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Health insurer / care</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>communityco@kp.org (Colorado community sponsorships, Sponsorship inbox (rules exclude advertising))</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr"/>
+          <t>kimpiet@iheartmedia.com (Kim Piet, Vice President of Partnerships)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>844-844-4432</t>
+        </is>
+      </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Email only</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>8</v>
+          <t>National ad sales line (sells ads). Ask for the Colorado Springs market president, Samantha Kumm, and pitch a media trade</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J24" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Paid sponsor of the Colorado Chamber’s 2024 pickleball tournament (Pickle Hour and awards) at the Broadmoor.</t>
-        </is>
-      </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Media partner, as above.</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>To find (statewide marketing; check for a Colorado Springs community contact)</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr"/>
-      <c r="P24" s="5" t="inlineStr"/>
+          <t>https://www.coloradospringssports.org/current-members</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>To find</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr"/>
       <c r="Q24" s="5" t="inlineStr"/>
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr"/>
-      <c r="U24" s="4" t="inlineStr"/>
-      <c r="V24" s="4" t="inlineStr"/>
+      <c r="U24" s="5" t="inlineStr"/>
+      <c r="V24" s="4" t="inlineStr">
+        <is>
+          <t>844-844-4432</t>
+        </is>
+      </c>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>national advertising line (no local number found); Colorado Springs Market President Samantha Kumm · https://www.iheartmedia.com/advertising</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -3145,63 +3238,68 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>OrangeTheory</t>
+          <t>Progressive</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Fitness</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>memberservices@orangetheory.com (General inbox)</t>
+          <t>chuck_jarrett@progressive.com (Charles Jarrett, Vice President And Chief Financial Officer)</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Email only</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>6</v>
+          <t>No good number (the ones found are the CFO and CEO). Email first; Colorado Springs campus has no public line</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H25" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>1</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Colorado Springs Sports Corp member, 2026 (Premier and Essential) tier: pays to back local sport. Fitness, not racquet sport: a cross-promotion partner more than a buyer.</t>
-        </is>
+      <c r="L25" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>https://www.coloradospringssports.org/current-members</t>
+          <t>Colorado Springs campus; about 1,500 staff in 2011 (old figure).</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>To find (franchise: the local owner decides)</t>
-        </is>
-      </c>
-      <c r="O25" s="4" t="inlineStr"/>
-      <c r="P25" s="5" t="inlineStr"/>
+          <t>Insurance Journal 2011 (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>To find (HR / benefits for memberships)</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr"/>
       <c r="Q25" s="5" t="inlineStr"/>
       <c r="R25" s="5" t="inlineStr"/>
       <c r="S25" s="5" t="inlineStr"/>
       <c r="T25" s="5" t="inlineStr"/>
-      <c r="U25" s="4" t="inlineStr"/>
+      <c r="U25" s="5" t="inlineStr"/>
       <c r="V25" s="4" t="inlineStr"/>
+      <c r="W25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -3209,63 +3307,68 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Chord Energy</t>
+          <t>USAA</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Insurance / banking</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>gilbert.delarosa@chordenergy.com (Gilbert Delarosa, Vice President of Marketing)</t>
+          <t>jennifer.escobar@usaa.com (Jennifer Escobar, VP of Brand Marketing)</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Email only</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>5</v>
+          <t>No good number (communications directors in other states). Email Jennifer Escobar, VP of Brand Marketing</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="J26" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
-        </is>
+      <c r="L26" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
+          <t>Large Colorado Springs campus; about 1,800 staff in 2017 (old figure). Military families: Peak’s neighbourhood.</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="5" t="inlineStr"/>
+          <t>Area Development 2017 (via search; see Fact-check)</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>To find (HR / benefits for memberships)</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr"/>
       <c r="Q26" s="5" t="inlineStr"/>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr"/>
-      <c r="U26" s="4" t="inlineStr"/>
+      <c r="U26" s="5" t="inlineStr"/>
       <c r="V26" s="4" t="inlineStr"/>
+      <c r="W26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -3287,49 +3390,50 @@
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Email only</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="n">
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="4" t="n">
+      <c r="I27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I27" s="4" t="n">
+      <c r="J27" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="4" t="n">
+      <c r="K27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K27" s="4" t="n">
+      <c r="L27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport. Host a member mixer at Peak.</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O27" s="4" t="inlineStr"/>
-      <c r="P27" s="5" t="inlineStr"/>
+      <c r="P27" s="4" t="inlineStr"/>
       <c r="Q27" s="5" t="inlineStr"/>
       <c r="R27" s="5" t="inlineStr"/>
       <c r="S27" s="5" t="inlineStr"/>
       <c r="T27" s="5" t="inlineStr"/>
-      <c r="U27" s="4" t="inlineStr"/>
+      <c r="U27" s="5" t="inlineStr"/>
       <c r="V27" s="4" t="inlineStr"/>
+      <c r="W27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -3351,49 +3455,50 @@
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Email only</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n">
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="4" t="n">
+      <c r="I28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="4" t="n">
+      <c r="J28" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="4" t="n">
+      <c r="K28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K28" s="4" t="n">
+      <c r="L28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Summit) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O28" s="4" t="inlineStr"/>
-      <c r="P28" s="5" t="inlineStr"/>
+      <c r="P28" s="4" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28" s="4" t="inlineStr"/>
+      <c r="U28" s="5" t="inlineStr"/>
       <c r="V28" s="4" t="inlineStr"/>
+      <c r="W28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -3415,49 +3520,50 @@
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Email only</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="n">
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Email first</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="I29" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O29" s="4" t="inlineStr"/>
-      <c r="P29" s="5" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr"/>
       <c r="R29" s="5" t="inlineStr"/>
       <c r="S29" s="5" t="inlineStr"/>
       <c r="T29" s="5" t="inlineStr"/>
-      <c r="U29" s="4" t="inlineStr"/>
+      <c r="U29" s="5" t="inlineStr"/>
       <c r="V29" s="4" t="inlineStr"/>
+      <c r="W29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -3475,49 +3581,50 @@
       </c>
       <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="H30" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H30" s="4" t="n">
+      <c r="I30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="4" t="n">
+      <c r="J30" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J30" s="4" t="n">
+      <c r="K30" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K30" s="4" t="n">
+      <c r="L30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>Court sponsor, Colorado Chamber 2024 pickleball tournament.</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="O30" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O30" s="4" t="inlineStr"/>
-      <c r="P30" s="5" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr"/>
       <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="inlineStr"/>
-      <c r="U30" s="4" t="inlineStr"/>
+      <c r="U30" s="5" t="inlineStr"/>
       <c r="V30" s="4" t="inlineStr"/>
+      <c r="W30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -3535,49 +3642,50 @@
       </c>
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="H31" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="J31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K31" s="4" t="n">
+      <c r="L31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>Court sponsor, Colorado Chamber 2024 pickleball tournament (name read from its web link; the logo text was unclear).</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>https://cochamber.com/event/2024-annual-pickleball-tournament</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="5" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr"/>
       <c r="Q31" s="5" t="inlineStr"/>
       <c r="R31" s="5" t="inlineStr"/>
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="inlineStr"/>
-      <c r="U31" s="4" t="inlineStr"/>
+      <c r="U31" s="5" t="inlineStr"/>
       <c r="V31" s="4" t="inlineStr"/>
+      <c r="W31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -3595,49 +3703,50 @@
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G32" s="4" t="n">
+      <c r="H32" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="I32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="J32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K32" s="4" t="n">
+      <c r="L32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="N32" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="O32" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O32" s="4" t="inlineStr"/>
-      <c r="P32" s="5" t="inlineStr"/>
+      <c r="P32" s="4" t="inlineStr"/>
       <c r="Q32" s="5" t="inlineStr"/>
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr"/>
       <c r="T32" s="5" t="inlineStr"/>
-      <c r="U32" s="4" t="inlineStr"/>
+      <c r="U32" s="5" t="inlineStr"/>
       <c r="V32" s="4" t="inlineStr"/>
+      <c r="W32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -3655,49 +3764,50 @@
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="H33" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H33" s="4" t="n">
+      <c r="I33" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="M33" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="O33" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O33" s="4" t="inlineStr"/>
-      <c r="P33" s="5" t="inlineStr"/>
+      <c r="P33" s="4" t="inlineStr"/>
       <c r="Q33" s="5" t="inlineStr"/>
       <c r="R33" s="5" t="inlineStr"/>
       <c r="S33" s="5" t="inlineStr"/>
       <c r="T33" s="5" t="inlineStr"/>
-      <c r="U33" s="4" t="inlineStr"/>
+      <c r="U33" s="5" t="inlineStr"/>
       <c r="V33" s="4" t="inlineStr"/>
+      <c r="W33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3715,49 +3825,50 @@
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G34" s="4" t="n">
+      <c r="H34" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H34" s="4" t="n">
+      <c r="I34" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="I34" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J34" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="M34" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O34" s="4" t="inlineStr"/>
-      <c r="P34" s="5" t="inlineStr"/>
+      <c r="P34" s="4" t="inlineStr"/>
       <c r="Q34" s="5" t="inlineStr"/>
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr"/>
       <c r="T34" s="5" t="inlineStr"/>
-      <c r="U34" s="4" t="inlineStr"/>
+      <c r="U34" s="5" t="inlineStr"/>
       <c r="V34" s="4" t="inlineStr"/>
+      <c r="W34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -3775,49 +3886,50 @@
       </c>
       <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="H35" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="I35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="4" t="n">
+      <c r="J35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J35" s="4" t="n">
+      <c r="K35" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K35" s="4" t="n">
+      <c r="L35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="M35" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Premier) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N35" s="4" t="inlineStr">
+      <c r="O35" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O35" s="4" t="inlineStr"/>
-      <c r="P35" s="5" t="inlineStr"/>
+      <c r="P35" s="4" t="inlineStr"/>
       <c r="Q35" s="5" t="inlineStr"/>
       <c r="R35" s="5" t="inlineStr"/>
       <c r="S35" s="5" t="inlineStr"/>
       <c r="T35" s="5" t="inlineStr"/>
-      <c r="U35" s="4" t="inlineStr"/>
+      <c r="U35" s="5" t="inlineStr"/>
       <c r="V35" s="4" t="inlineStr"/>
+      <c r="W35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3835,49 +3947,50 @@
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G36" s="4" t="n">
+      <c r="H36" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H36" s="4" t="n">
+      <c r="I36" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I36" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="M36" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="O36" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O36" s="4" t="inlineStr"/>
-      <c r="P36" s="5" t="inlineStr"/>
+      <c r="P36" s="4" t="inlineStr"/>
       <c r="Q36" s="5" t="inlineStr"/>
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr"/>
       <c r="T36" s="5" t="inlineStr"/>
-      <c r="U36" s="4" t="inlineStr"/>
+      <c r="U36" s="5" t="inlineStr"/>
       <c r="V36" s="4" t="inlineStr"/>
+      <c r="W36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3895,49 +4008,50 @@
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G37" s="4" t="n">
+      <c r="H37" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H37" s="4" t="n">
+      <c r="I37" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I37" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="M37" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N37" s="4" t="inlineStr">
+      <c r="O37" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O37" s="4" t="inlineStr"/>
-      <c r="P37" s="5" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr"/>
       <c r="Q37" s="5" t="inlineStr"/>
       <c r="R37" s="5" t="inlineStr"/>
       <c r="S37" s="5" t="inlineStr"/>
       <c r="T37" s="5" t="inlineStr"/>
-      <c r="U37" s="4" t="inlineStr"/>
+      <c r="U37" s="5" t="inlineStr"/>
       <c r="V37" s="4" t="inlineStr"/>
+      <c r="W37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -3955,49 +4069,50 @@
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr"/>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G38" s="4" t="n">
+      <c r="H38" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H38" s="4" t="n">
+      <c r="I38" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I38" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="M38" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport. Family audience.</t>
         </is>
       </c>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N38" s="4" t="inlineStr">
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O38" s="4" t="inlineStr"/>
-      <c r="P38" s="5" t="inlineStr"/>
+      <c r="P38" s="4" t="inlineStr"/>
       <c r="Q38" s="5" t="inlineStr"/>
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr"/>
       <c r="T38" s="5" t="inlineStr"/>
-      <c r="U38" s="4" t="inlineStr"/>
+      <c r="U38" s="5" t="inlineStr"/>
       <c r="V38" s="4" t="inlineStr"/>
+      <c r="W38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -4015,49 +4130,50 @@
       </c>
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G39" s="4" t="n">
+      <c r="H39" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H39" s="4" t="n">
+      <c r="I39" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I39" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L39" s="4" t="inlineStr">
+      <c r="M39" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M39" s="4" t="inlineStr">
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N39" s="4" t="inlineStr">
+      <c r="O39" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O39" s="4" t="inlineStr"/>
-      <c r="P39" s="5" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr"/>
       <c r="R39" s="5" t="inlineStr"/>
       <c r="S39" s="5" t="inlineStr"/>
       <c r="T39" s="5" t="inlineStr"/>
-      <c r="U39" s="4" t="inlineStr"/>
+      <c r="U39" s="5" t="inlineStr"/>
       <c r="V39" s="4" t="inlineStr"/>
+      <c r="W39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -4075,54 +4191,55 @@
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>Neither yet</t>
         </is>
       </c>
-      <c r="G40" s="4" t="n">
+      <c r="H40" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="4" t="n">
+      <c r="I40" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="I40" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="J40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L40" s="4" t="inlineStr">
+      <c r="M40" s="4" t="inlineStr">
         <is>
           <t>Colorado Springs Sports Corp member, 2026 (Essential) tier: pays to back local sport.</t>
         </is>
       </c>
-      <c r="M40" s="4" t="inlineStr">
+      <c r="N40" s="4" t="inlineStr">
         <is>
           <t>https://www.coloradospringssports.org/current-members</t>
         </is>
       </c>
-      <c r="N40" s="4" t="inlineStr">
+      <c r="O40" s="4" t="inlineStr">
         <is>
           <t>To find</t>
         </is>
       </c>
-      <c r="O40" s="4" t="inlineStr"/>
-      <c r="P40" s="5" t="inlineStr"/>
+      <c r="P40" s="4" t="inlineStr"/>
       <c r="Q40" s="5" t="inlineStr"/>
       <c r="R40" s="5" t="inlineStr"/>
       <c r="S40" s="5" t="inlineStr"/>
       <c r="T40" s="5" t="inlineStr"/>
-      <c r="U40" s="4" t="inlineStr"/>
+      <c r="U40" s="5" t="inlineStr"/>
       <c r="V40" s="4" t="inlineStr"/>
+      <c r="W40" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V40"/>
+  <autoFilter ref="A1:W40"/>
   <dataValidations count="1">
-    <dataValidation sqref="P2:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,Emailed,Called,Tour booked,Toured,Proposal sent,Signed,Not now,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>